<commit_message>
Clarify per-rank inference capacity fields
</commit_message>
<xml_diff>
--- a/calculate/deepseek_v4_flash_calculator.xlsx
+++ b/calculate/deepseek_v4_flash_calculator.xlsx
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1128" uniqueCount="603">
   <si>
     <t>DeepSeek V4 Flash - Editable Architecture Parameters</t>
   </si>
@@ -1753,25 +1753,34 @@
     <t>Decode TP8 GB</t>
   </si>
   <si>
-    <t>TP1 参数 GB/rank</t>
-  </si>
-  <si>
-    <t>TP8 参数 GB/rank</t>
-  </si>
-  <si>
-    <t>容量项</t>
-  </si>
-  <si>
-    <t>TP1 GB/rank</t>
-  </si>
-  <si>
-    <t>TP8 GB/rank</t>
-  </si>
-  <si>
-    <t>参数</t>
-  </si>
-  <si>
-    <t>Decode KV+State</t>
+    <t>静态参数大类（Prefill/Decode 共用）</t>
+  </si>
+  <si>
+    <t>TP1 单 Rank GB</t>
+  </si>
+  <si>
+    <t>TP8 单 Rank GB</t>
+  </si>
+  <si>
+    <t>说明：参数容量只由模型结构、dtype 和 TP 分片决定，与 Prefill/Decode 场景无关；两列分别是单 Rank 值，不相加。</t>
+  </si>
+  <si>
+    <t>推理场景容量项</t>
+  </si>
+  <si>
+    <t>静态参数（场景共用）</t>
+  </si>
+  <si>
+    <t>Prefill 预分配 KV+State</t>
+  </si>
+  <si>
+    <t>Prefill 总驻留（参数+KV）</t>
+  </si>
+  <si>
+    <t>Decode 预分配 KV+State</t>
+  </si>
+  <si>
+    <t>Decode 总驻留（参数+KV）</t>
   </si>
   <si>
     <t>方法与统计边界</t>
@@ -2936,7 +2945,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>每 Rank 参数容量</a:t>
+              <a:t>静态参数容量/单 Rank（Prefill/Decode 共用）</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2952,7 +2961,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>TP1</c:v>
+            <c:v>TP1 单 Rank</c:v>
           </c:tx>
           <c:dLbls>
             <c:numFmt formatCode="0.0" sourceLinked="0"/>
@@ -2998,7 +3007,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>TP8</c:v>
+            <c:v>TP8 单 Rank</c:v>
           </c:tx>
           <c:dLbls>
             <c:numFmt formatCode="0.0" sourceLinked="0"/>
@@ -3118,7 +3127,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Decode 每 Rank 驻留容量</a:t>
+              <a:t>Prefill / Decode 单 Rank 容量（TP 配置独立）</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -3134,7 +3143,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>TP1</c:v>
+            <c:v>TP1 单 Rank</c:v>
           </c:tx>
           <c:dLbls>
             <c:numFmt formatCode="0.0" sourceLinked="0"/>
@@ -3142,29 +3151,47 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Comparison!$A$23:$A$24</c:f>
+              <c:f>Comparison!$A$23:$A$27</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>参数</c:v>
+                  <c:v>静态参数（场景共用）</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Decode KV+State</c:v>
+                  <c:v>Prefill 预分配 KV+State</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Prefill 总驻留（参数+KV）</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Decode 预分配 KV+State</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Decode 总驻留（参数+KV）</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Comparison!$B$23:$B$24</c:f>
+              <c:f>Comparison!$B$23:$B$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>159.117270492</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>7.232045056</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>166.349315548</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.232045056</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>166.349315548</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3174,7 +3201,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>TP8</c:v>
+            <c:v>TP8 单 Rank</c:v>
           </c:tx>
           <c:dLbls>
             <c:numFmt formatCode="0.0" sourceLinked="0"/>
@@ -3182,29 +3209,47 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Comparison!$A$23:$A$24</c:f>
+              <c:f>Comparison!$A$23:$A$27</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>参数</c:v>
+                  <c:v>静态参数（场景共用）</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Decode KV+State</c:v>
+                  <c:v>Prefill 预分配 KV+State</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Prefill 总驻留（参数+KV）</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Decode 预分配 KV+State</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Decode 总驻留（参数+KV）</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Comparison!$C$23:$C$24</c:f>
+              <c:f>Comparison!$C$23:$C$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>22.349822332</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>7.232045056</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>29.581867388</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.232045056</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>29.581867388</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12419,7 +12464,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -12598,13 +12643,13 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="3" t="s">
-        <v>404</v>
+        <v>517</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -12646,15 +12691,20 @@
         <v>0.534376892</v>
       </c>
     </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="2" t="s">
+        <v>520</v>
+      </c>
+    </row>
     <row r="22" spans="1:3">
       <c r="A22" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>519</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>520</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -12675,12 +12725,51 @@
         <v>523</v>
       </c>
       <c r="B24" s="13">
+        <f>'Memory'!$P$29/1E9</f>
+        <v>7.232045056</v>
+      </c>
+      <c r="C24" s="13">
+        <f>'Memory'!$Q$29/1E9</f>
+        <v>7.232045056</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B25" s="13">
+        <f>'Memory'!$R$21+'Memory'!$P$29/1E9</f>
+        <v>166.349315548</v>
+      </c>
+      <c r="C25" s="13">
+        <f>'Memory'!$S$21+'Memory'!$Q$29/1E9</f>
+        <v>29.581867388</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="B26" s="13">
         <f>'Memory'!$P$33/1E9</f>
         <v>7.232045056</v>
       </c>
-      <c r="C24" s="13">
+      <c r="C26" s="13">
         <f>'Memory'!$Q$33/1E9</f>
         <v>7.232045056</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="B27" s="13">
+        <f>'Memory'!$R$21+'Memory'!$P$33/1E9</f>
+        <v>166.349315548</v>
+      </c>
+      <c r="C27" s="13">
+        <f>'Memory'!$S$21+'Memory'!$Q$33/1E9</f>
+        <v>29.581867388</v>
       </c>
     </row>
   </sheetData>
@@ -12700,47 +12789,47 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="3" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="4" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="4" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="4" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="4" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -12748,55 +12837,55 @@
         <v>67</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="4" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="4" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="4" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="4" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -12804,15 +12893,15 @@
         <v>460</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
     </row>
   </sheetData>
@@ -12833,17 +12922,17 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="7" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -12853,16 +12942,16 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>460</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>460</v>
@@ -12873,7 +12962,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="4" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="B6" s="12">
         <f>IF(ABS(G6)&gt;=1E15,G6/1E15,IF(ABS(G6)&gt;=1E12,G6/1E12,IF(ABS(G6)&gt;=1E9,G6/1E9,IF(ABS(G6)&gt;=1E6,G6/1E6,G6))))</f>
@@ -12892,7 +12981,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="G6" s="13">
         <f>'Prefill_8K'!$AE$13</f>
@@ -12905,7 +12994,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="4" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="B7" s="12">
         <f>IF(ABS(G7)&gt;=1E15,G7/1E15,IF(ABS(G7)&gt;=1E12,G7/1E12,IF(ABS(G7)&gt;=1E9,G7/1E9,IF(ABS(G7)&gt;=1E6,G7/1E6,G7))))</f>
@@ -12924,7 +13013,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="G7" s="13">
         <f>'Prefill_8K'!$AE$14</f>
@@ -12937,7 +13026,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="4" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B8" s="12">
         <f>IF(ABS(G8)&gt;=1E15,G8/1E15,IF(ABS(G8)&gt;=1E12,G8/1E12,IF(ABS(G8)&gt;=1E9,G8/1E9,IF(ABS(G8)&gt;=1E6,G8/1E6,G8))))</f>
@@ -12956,7 +13045,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="G8" s="13">
         <f>'Prefill_8K'!$AE$15</f>
@@ -12969,7 +13058,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="14" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="B9" s="14">
         <f>IF(ABS(G9)&gt;=1E15,G9/1E15,IF(ABS(G9)&gt;=1E12,G9/1E12,IF(ABS(G9)&gt;=1E9,G9/1E9,IF(ABS(G9)&gt;=1E6,G9/1E6,G9))))</f>
@@ -12988,7 +13077,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="G9" s="13">
         <f>'Prefill_8K'!$AE$16</f>
@@ -13001,7 +13090,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="4" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B10" s="12">
         <f>IF(ABS(G10)&gt;=1E12,G10/1E12,IF(ABS(G10)&gt;=1E9,G10/1E9,IF(ABS(G10)&gt;=1E6,G10/1E6,IF(ABS(G10)&gt;=1E3,G10/1E3,G10))))</f>
@@ -13020,7 +13109,7 @@
         <v>GB</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="G10" s="13">
         <f>'Prefill_8K'!$AE$17</f>
@@ -13033,7 +13122,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="4" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B11" s="12">
         <f>IF(ABS(G11)&gt;=1E12,G11/1E12,IF(ABS(G11)&gt;=1E9,G11/1E9,IF(ABS(G11)&gt;=1E6,G11/1E6,IF(ABS(G11)&gt;=1E3,G11/1E3,G11))))</f>
@@ -13052,7 +13141,7 @@
         <v>GB</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="G11" s="13">
         <f>'Prefill_8K'!$AE$18</f>
@@ -13065,7 +13154,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="4" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B12" s="12">
         <f>IF(ABS(G12)&gt;=1E12,G12/1E12,IF(ABS(G12)&gt;=1E9,G12/1E9,IF(ABS(G12)&gt;=1E6,G12/1E6,IF(ABS(G12)&gt;=1E3,G12/1E3,G12))))</f>
@@ -13084,7 +13173,7 @@
         <v>GB</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="G12" s="13">
         <f>'Prefill_8K'!$AE$19</f>
@@ -13097,7 +13186,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="14" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B13" s="14">
         <f>IF(ABS(G13)&gt;=1E12,G13/1E12,IF(ABS(G13)&gt;=1E9,G13/1E9,IF(ABS(G13)&gt;=1E6,G13/1E6,IF(ABS(G13)&gt;=1E3,G13/1E3,G13))))</f>
@@ -13116,7 +13205,7 @@
         <v>GB</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="G13" s="13">
         <f>'Prefill_8K'!$AE$20</f>
@@ -13129,7 +13218,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="4" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="B14" s="12">
         <f>G14</f>
@@ -13146,7 +13235,7 @@
         <v>159</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="G14" s="13">
         <f>'Prefill_8K'!$AE$17/(PrefillTargetMs/1000)/1E9</f>
@@ -13159,7 +13248,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="4" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B15" s="12">
         <f>G15</f>
@@ -13176,7 +13265,7 @@
         <v>159</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="G15" s="13">
         <f>'Prefill_8K'!$AE$18/(PrefillTargetMs/1000)/1E9</f>
@@ -13189,7 +13278,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="4" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="B16" s="12">
         <f>G16</f>
@@ -13206,7 +13295,7 @@
         <v>159</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="G16" s="13">
         <f>'Prefill_8K'!$AE$19/(PrefillTargetMs/1000)/1E9</f>
@@ -13219,7 +13308,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="4" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B17" s="12">
         <f>G17</f>
@@ -13236,7 +13325,7 @@
         <v>155</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="G17" s="13">
         <f>'Prefill_8K'!$AE$23</f>
@@ -13249,7 +13338,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="4" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="B18" s="12">
         <f>IF(ABS(G18)&gt;=1E12,G18/1E12,IF(ABS(G18)&gt;=1E9,G18/1E9,IF(ABS(G18)&gt;=1E6,G18/1E6,IF(ABS(G18)&gt;=1E3,G18/1E3,G18))))</f>
@@ -13268,7 +13357,7 @@
         <v>B</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="G18" s="13">
         <f>'Prefill_8K'!$AE$21</f>
@@ -13281,7 +13370,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="4" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="B19" s="12">
         <f>G19</f>
@@ -13298,7 +13387,7 @@
         <v>159</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="G19" s="13">
         <f>'Prefill_8K'!$AE$21/(PrefillTargetMs/1000)/1E9</f>
@@ -13311,7 +13400,7 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="4" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B20" s="12">
         <f>IF(ABS(G20)&gt;=1E12,G20/1E12,IF(ABS(G20)&gt;=1E9,G20/1E9,IF(ABS(G20)&gt;=1E6,G20/1E6,IF(ABS(G20)&gt;=1E3,G20/1E3,G20))))</f>
@@ -13330,7 +13419,7 @@
         <v>G params</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="G20" s="13">
         <f>'Memory'!$P$18</f>
@@ -13343,7 +13432,7 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="4" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="B21" s="12">
         <f>IF(ABS(G21)&gt;=1E12,G21/1E12,IF(ABS(G21)&gt;=1E9,G21/1E9,IF(ABS(G21)&gt;=1E6,G21/1E6,IF(ABS(G21)&gt;=1E3,G21/1E3,G21))))</f>
@@ -13362,7 +13451,7 @@
         <v>G params</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="G21" s="13">
         <f>'Memory'!$P$19</f>
@@ -13375,7 +13464,7 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="4" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B22" s="12">
         <f>IF(ABS(G22)&gt;=1E12,G22/1E12,IF(ABS(G22)&gt;=1E9,G22/1E9,IF(ABS(G22)&gt;=1E6,G22/1E6,IF(ABS(G22)&gt;=1E3,G22/1E3,G22))))</f>
@@ -13394,7 +13483,7 @@
         <v>G params</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="G22" s="13">
         <f>'Memory'!$P$20</f>
@@ -13407,7 +13496,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="14" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="B23" s="14">
         <f>IF(ABS(G23)&gt;=1E12,G23/1E12,IF(ABS(G23)&gt;=1E9,G23/1E9,IF(ABS(G23)&gt;=1E6,G23/1E6,IF(ABS(G23)&gt;=1E3,G23/1E3,G23))))</f>
@@ -13426,7 +13515,7 @@
         <v>G params</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="G23" s="13">
         <f>'Memory'!$P$21</f>
@@ -13439,7 +13528,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="4" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="B24" s="12">
         <f>IF(ABS(G24)&gt;=1E12,G24/1E12,IF(ABS(G24)&gt;=1E9,G24/1E9,IF(ABS(G24)&gt;=1E6,G24/1E6,IF(ABS(G24)&gt;=1E3,G24/1E3,G24))))</f>
@@ -13458,7 +13547,7 @@
         <v>GB</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="G24" s="13">
         <f>'Memory'!$R$18</f>
@@ -13471,7 +13560,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="4" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="B25" s="12">
         <f>IF(ABS(G25)&gt;=1E12,G25/1E12,IF(ABS(G25)&gt;=1E9,G25/1E9,IF(ABS(G25)&gt;=1E6,G25/1E6,IF(ABS(G25)&gt;=1E3,G25/1E3,G25))))</f>
@@ -13490,7 +13579,7 @@
         <v>GB</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="G25" s="13">
         <f>'Memory'!$R$19</f>
@@ -13503,7 +13592,7 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="4" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="B26" s="12">
         <f>IF(ABS(G26)&gt;=1E12,G26/1E12,IF(ABS(G26)&gt;=1E9,G26/1E9,IF(ABS(G26)&gt;=1E6,G26/1E6,IF(ABS(G26)&gt;=1E3,G26/1E3,G26))))</f>
@@ -13522,7 +13611,7 @@
         <v>GB</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="G26" s="13">
         <f>'Memory'!$R$20</f>
@@ -13535,7 +13624,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="14" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B27" s="14">
         <f>IF(ABS(G27)&gt;=1E12,G27/1E12,IF(ABS(G27)&gt;=1E9,G27/1E9,IF(ABS(G27)&gt;=1E6,G27/1E6,IF(ABS(G27)&gt;=1E3,G27/1E3,G27))))</f>
@@ -13554,7 +13643,7 @@
         <v>GB</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="G27" s="13">
         <f>'Memory'!$R$21</f>
@@ -13567,7 +13656,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="4" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="B28" s="12">
         <f>IF(ABS(G28)&gt;=1E12,G28/1E12,IF(ABS(G28)&gt;=1E9,G28/1E9,IF(ABS(G28)&gt;=1E6,G28/1E6,IF(ABS(G28)&gt;=1E3,G28/1E3,G28))))</f>
@@ -13586,7 +13675,7 @@
         <v>GB</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G28" s="13">
         <f>'Memory'!$P$26</f>
@@ -13599,7 +13688,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="4" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B29" s="12">
         <f>IF(ABS(G29)&gt;=1E12,G29/1E12,IF(ABS(G29)&gt;=1E9,G29/1E9,IF(ABS(G29)&gt;=1E6,G29/1E6,IF(ABS(G29)&gt;=1E3,G29/1E3,G29))))</f>
@@ -13618,7 +13707,7 @@
         <v>GB</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G29" s="13">
         <f>'Memory'!$P$27</f>
@@ -13631,7 +13720,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="4" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="B30" s="12">
         <f>IF(ABS(G30)&gt;=1E12,G30/1E12,IF(ABS(G30)&gt;=1E9,G30/1E9,IF(ABS(G30)&gt;=1E6,G30/1E6,IF(ABS(G30)&gt;=1E3,G30/1E3,G30))))</f>
@@ -13650,7 +13739,7 @@
         <v>MB</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G30" s="13">
         <f>'Memory'!$P$28</f>
@@ -13663,7 +13752,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="4" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="B31" s="12">
         <f>IF(ABS(G31)&gt;=1E12,G31/1E12,IF(ABS(G31)&gt;=1E9,G31/1E9,IF(ABS(G31)&gt;=1E6,G31/1E6,IF(ABS(G31)&gt;=1E3,G31/1E3,G31))))</f>
@@ -13682,7 +13771,7 @@
         <v>GB</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G31" s="13">
         <f>'Memory'!$P$29</f>
@@ -13695,7 +13784,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="14" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="B32" s="14">
         <f>IF(ABS(G32)&gt;=1E12,G32/1E12,IF(ABS(G32)&gt;=1E9,G32/1E9,IF(ABS(G32)&gt;=1E6,G32/1E6,IF(ABS(G32)&gt;=1E3,G32/1E3,G32))))</f>
@@ -13714,7 +13803,7 @@
         <v>GB</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="G32" s="13">
         <f>'Memory'!$R$21+'Memory'!$P$29</f>
@@ -13727,7 +13816,7 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="7" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
@@ -13737,16 +13826,16 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="3" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>460</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>460</v>
@@ -13757,7 +13846,7 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="4" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="B36" s="12">
         <f>IF(ABS(G36)&gt;=1E15,G36/1E15,IF(ABS(G36)&gt;=1E12,G36/1E12,IF(ABS(G36)&gt;=1E9,G36/1E9,IF(ABS(G36)&gt;=1E6,G36/1E6,G36))))</f>
@@ -13776,7 +13865,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="G36" s="13">
         <f>'Prefill_8K'!$AF$13</f>
@@ -13789,7 +13878,7 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="4" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="B37" s="12">
         <f>IF(ABS(G37)&gt;=1E15,G37/1E15,IF(ABS(G37)&gt;=1E12,G37/1E12,IF(ABS(G37)&gt;=1E9,G37/1E9,IF(ABS(G37)&gt;=1E6,G37/1E6,G37))))</f>
@@ -13808,7 +13897,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="G37" s="13">
         <f>'Prefill_8K'!$AF$14</f>
@@ -13821,7 +13910,7 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="4" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B38" s="12">
         <f>IF(ABS(G38)&gt;=1E15,G38/1E15,IF(ABS(G38)&gt;=1E12,G38/1E12,IF(ABS(G38)&gt;=1E9,G38/1E9,IF(ABS(G38)&gt;=1E6,G38/1E6,G38))))</f>
@@ -13840,7 +13929,7 @@
         <v>MFLOPs</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="G38" s="13">
         <f>'Prefill_8K'!$AF$15</f>
@@ -13853,7 +13942,7 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="14" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="B39" s="14">
         <f>IF(ABS(G39)&gt;=1E15,G39/1E15,IF(ABS(G39)&gt;=1E12,G39/1E12,IF(ABS(G39)&gt;=1E9,G39/1E9,IF(ABS(G39)&gt;=1E6,G39/1E6,G39))))</f>
@@ -13872,7 +13961,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="G39" s="13">
         <f>'Prefill_8K'!$AF$16</f>
@@ -13885,7 +13974,7 @@
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="4" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B40" s="12">
         <f>IF(ABS(G40)&gt;=1E12,G40/1E12,IF(ABS(G40)&gt;=1E9,G40/1E9,IF(ABS(G40)&gt;=1E6,G40/1E6,IF(ABS(G40)&gt;=1E3,G40/1E3,G40))))</f>
@@ -13904,7 +13993,7 @@
         <v>GB</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="G40" s="13">
         <f>'Prefill_8K'!$AF$17</f>
@@ -13917,7 +14006,7 @@
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="4" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B41" s="12">
         <f>IF(ABS(G41)&gt;=1E12,G41/1E12,IF(ABS(G41)&gt;=1E9,G41/1E9,IF(ABS(G41)&gt;=1E6,G41/1E6,IF(ABS(G41)&gt;=1E3,G41/1E3,G41))))</f>
@@ -13936,7 +14025,7 @@
         <v>GB</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="G41" s="13">
         <f>'Prefill_8K'!$AF$18</f>
@@ -13949,7 +14038,7 @@
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="4" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B42" s="12">
         <f>IF(ABS(G42)&gt;=1E12,G42/1E12,IF(ABS(G42)&gt;=1E9,G42/1E9,IF(ABS(G42)&gt;=1E6,G42/1E6,IF(ABS(G42)&gt;=1E3,G42/1E3,G42))))</f>
@@ -13968,7 +14057,7 @@
         <v>MB</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="G42" s="13">
         <f>'Prefill_8K'!$AF$19</f>
@@ -13981,7 +14070,7 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="14" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B43" s="14">
         <f>IF(ABS(G43)&gt;=1E12,G43/1E12,IF(ABS(G43)&gt;=1E9,G43/1E9,IF(ABS(G43)&gt;=1E6,G43/1E6,IF(ABS(G43)&gt;=1E3,G43/1E3,G43))))</f>
@@ -14000,7 +14089,7 @@
         <v>GB</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="G43" s="13">
         <f>'Prefill_8K'!$AF$20</f>
@@ -14013,7 +14102,7 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="4" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="B44" s="12">
         <f>G44</f>
@@ -14030,7 +14119,7 @@
         <v>159</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="G44" s="13">
         <f>'Prefill_8K'!$AF$17/(PrefillTargetMs/1000)/1E9</f>
@@ -14043,7 +14132,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="4" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B45" s="12">
         <f>G45</f>
@@ -14060,7 +14149,7 @@
         <v>159</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="G45" s="13">
         <f>'Prefill_8K'!$AF$18/(PrefillTargetMs/1000)/1E9</f>
@@ -14073,7 +14162,7 @@
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="4" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="B46" s="12">
         <f>G46</f>
@@ -14090,7 +14179,7 @@
         <v>159</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="G46" s="13">
         <f>'Prefill_8K'!$AF$19/(PrefillTargetMs/1000)/1E9</f>
@@ -14103,7 +14192,7 @@
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="4" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B47" s="12">
         <f>G47</f>
@@ -14120,7 +14209,7 @@
         <v>155</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="G47" s="13">
         <f>'Prefill_8K'!$AF$23</f>
@@ -14133,7 +14222,7 @@
     </row>
     <row r="48" spans="1:8">
       <c r="A48" s="4" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="B48" s="12">
         <f>IF(ABS(G48)&gt;=1E12,G48/1E12,IF(ABS(G48)&gt;=1E9,G48/1E9,IF(ABS(G48)&gt;=1E6,G48/1E6,IF(ABS(G48)&gt;=1E3,G48/1E3,G48))))</f>
@@ -14152,7 +14241,7 @@
         <v>MB</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="G48" s="13">
         <f>'Prefill_8K'!$AF$21</f>
@@ -14165,7 +14254,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="4" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="B49" s="12">
         <f>G49</f>
@@ -14182,7 +14271,7 @@
         <v>159</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="G49" s="13">
         <f>'Prefill_8K'!$AF$21/(PrefillTargetMs/1000)/1E9</f>
@@ -14195,7 +14284,7 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="4" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B50" s="12">
         <f>IF(ABS(G50)&gt;=1E12,G50/1E12,IF(ABS(G50)&gt;=1E9,G50/1E9,IF(ABS(G50)&gt;=1E6,G50/1E6,IF(ABS(G50)&gt;=1E3,G50/1E3,G50))))</f>
@@ -14214,7 +14303,7 @@
         <v>G params</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="G50" s="13">
         <f>'Memory'!$Q$18</f>
@@ -14227,7 +14316,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="4" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="B51" s="12">
         <f>IF(ABS(G51)&gt;=1E12,G51/1E12,IF(ABS(G51)&gt;=1E9,G51/1E9,IF(ABS(G51)&gt;=1E6,G51/1E6,IF(ABS(G51)&gt;=1E3,G51/1E3,G51))))</f>
@@ -14246,7 +14335,7 @@
         <v>G params</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="G51" s="13">
         <f>'Memory'!$Q$19</f>
@@ -14259,7 +14348,7 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="4" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B52" s="12">
         <f>IF(ABS(G52)&gt;=1E12,G52/1E12,IF(ABS(G52)&gt;=1E9,G52/1E9,IF(ABS(G52)&gt;=1E6,G52/1E6,IF(ABS(G52)&gt;=1E3,G52/1E3,G52))))</f>
@@ -14278,7 +14367,7 @@
         <v>M params</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="G52" s="13">
         <f>'Memory'!$Q$20</f>
@@ -14291,7 +14380,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="14" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="B53" s="14">
         <f>IF(ABS(G53)&gt;=1E12,G53/1E12,IF(ABS(G53)&gt;=1E9,G53/1E9,IF(ABS(G53)&gt;=1E6,G53/1E6,IF(ABS(G53)&gt;=1E3,G53/1E3,G53))))</f>
@@ -14310,7 +14399,7 @@
         <v>G params</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="G53" s="13">
         <f>'Memory'!$Q$21</f>
@@ -14323,7 +14412,7 @@
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="4" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="B54" s="12">
         <f>IF(ABS(G54)&gt;=1E12,G54/1E12,IF(ABS(G54)&gt;=1E9,G54/1E9,IF(ABS(G54)&gt;=1E6,G54/1E6,IF(ABS(G54)&gt;=1E3,G54/1E3,G54))))</f>
@@ -14342,7 +14431,7 @@
         <v>GB</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="G54" s="13">
         <f>'Memory'!$S$18</f>
@@ -14355,7 +14444,7 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="4" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="B55" s="12">
         <f>IF(ABS(G55)&gt;=1E12,G55/1E12,IF(ABS(G55)&gt;=1E9,G55/1E9,IF(ABS(G55)&gt;=1E6,G55/1E6,IF(ABS(G55)&gt;=1E3,G55/1E3,G55))))</f>
@@ -14374,7 +14463,7 @@
         <v>GB</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="G55" s="13">
         <f>'Memory'!$S$19</f>
@@ -14387,7 +14476,7 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="4" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="B56" s="12">
         <f>IF(ABS(G56)&gt;=1E12,G56/1E12,IF(ABS(G56)&gt;=1E9,G56/1E9,IF(ABS(G56)&gt;=1E6,G56/1E6,IF(ABS(G56)&gt;=1E3,G56/1E3,G56))))</f>
@@ -14406,7 +14495,7 @@
         <v>MB</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="G56" s="13">
         <f>'Memory'!$S$20</f>
@@ -14419,7 +14508,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="14" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B57" s="14">
         <f>IF(ABS(G57)&gt;=1E12,G57/1E12,IF(ABS(G57)&gt;=1E9,G57/1E9,IF(ABS(G57)&gt;=1E6,G57/1E6,IF(ABS(G57)&gt;=1E3,G57/1E3,G57))))</f>
@@ -14438,7 +14527,7 @@
         <v>GB</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="G57" s="13">
         <f>'Memory'!$S$21</f>
@@ -14451,7 +14540,7 @@
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="4" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="B58" s="12">
         <f>IF(ABS(G58)&gt;=1E12,G58/1E12,IF(ABS(G58)&gt;=1E9,G58/1E9,IF(ABS(G58)&gt;=1E6,G58/1E6,IF(ABS(G58)&gt;=1E3,G58/1E3,G58))))</f>
@@ -14470,7 +14559,7 @@
         <v>GB</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G58" s="13">
         <f>'Memory'!$Q$26</f>
@@ -14483,7 +14572,7 @@
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="4" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B59" s="12">
         <f>IF(ABS(G59)&gt;=1E12,G59/1E12,IF(ABS(G59)&gt;=1E9,G59/1E9,IF(ABS(G59)&gt;=1E6,G59/1E6,IF(ABS(G59)&gt;=1E3,G59/1E3,G59))))</f>
@@ -14502,7 +14591,7 @@
         <v>GB</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G59" s="13">
         <f>'Memory'!$Q$27</f>
@@ -14515,7 +14604,7 @@
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="4" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="B60" s="12">
         <f>IF(ABS(G60)&gt;=1E12,G60/1E12,IF(ABS(G60)&gt;=1E9,G60/1E9,IF(ABS(G60)&gt;=1E6,G60/1E6,IF(ABS(G60)&gt;=1E3,G60/1E3,G60))))</f>
@@ -14534,7 +14623,7 @@
         <v>MB</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G60" s="13">
         <f>'Memory'!$Q$28</f>
@@ -14547,7 +14636,7 @@
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="4" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="B61" s="12">
         <f>IF(ABS(G61)&gt;=1E12,G61/1E12,IF(ABS(G61)&gt;=1E9,G61/1E9,IF(ABS(G61)&gt;=1E6,G61/1E6,IF(ABS(G61)&gt;=1E3,G61/1E3,G61))))</f>
@@ -14566,7 +14655,7 @@
         <v>GB</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G61" s="13">
         <f>'Memory'!$Q$29</f>
@@ -14579,7 +14668,7 @@
     </row>
     <row r="62" spans="1:8">
       <c r="A62" s="14" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="B62" s="14">
         <f>IF(ABS(G62)&gt;=1E12,G62/1E12,IF(ABS(G62)&gt;=1E9,G62/1E9,IF(ABS(G62)&gt;=1E6,G62/1E6,IF(ABS(G62)&gt;=1E3,G62/1E3,G62))))</f>
@@ -14598,7 +14687,7 @@
         <v>GB</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="G62" s="13">
         <f>'Memory'!$S$21+'Memory'!$Q$29</f>

</xml_diff>

<commit_message>
Rearrange comparison charts and units
</commit_message>
<xml_diff>
--- a/calculate/deepseek_v4_flash_calculator.xlsx
+++ b/calculate/deepseek_v4_flash_calculator.xlsx
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1128" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="609">
   <si>
     <t>DeepSeek V4 Flash - Editable Architecture Parameters</t>
   </si>
@@ -1781,6 +1781,24 @@
   </si>
   <si>
     <t>Decode 总驻留（参数+KV）</t>
+  </si>
+  <si>
+    <t>算力需求场景</t>
+  </si>
+  <si>
+    <t>所需 TFLOP/s</t>
+  </si>
+  <si>
+    <t>Prefill TP1/rank</t>
+  </si>
+  <si>
+    <t>Prefill TP8/rank</t>
+  </si>
+  <si>
+    <t>Decode TP1/rank</t>
+  </si>
+  <si>
+    <t>Decode TP8/rank</t>
   </si>
   <si>
     <t>方法与统计边界</t>
@@ -2217,6 +2235,148 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
+              <a:t>目标时延所需总算力/单 Rank</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>所需 TFLOP/s</c:v>
+          </c:tx>
+          <c:dLbls>
+            <c:numFmt formatCode="0.0" sourceLinked="0"/>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Comparison!$A$31:$A$34</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Prefill TP1/rank</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Prefill TP8/rank</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Decode TP1/rank</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Decode TP8/rank</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Comparison!$B$31:$B$34</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>228.384427393024</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>55.63931418624</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>14.0354134102</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.3548076118</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="low"/>
+        <c:crossAx val="50010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>TFLOP/s</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:style val="10"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
               <a:t>Prefill 每 Rank 计算量</a:t>
             </a:r>
           </a:p>
@@ -2321,24 +2481,24 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50010001"/>
-        <c:axId val="50010002"/>
+        <c:axId val="50020001"/>
+        <c:axId val="50020002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50010001"/>
+        <c:axId val="50020001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="50010002"/>
+        <c:crossAx val="50020002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50010002"/>
+        <c:axId val="50020002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2364,7 +2524,7 @@
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50010001"/>
+        <c:crossAx val="50020001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2383,7 +2543,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:style val="10"/>
@@ -2503,24 +2663,24 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50020001"/>
-        <c:axId val="50020002"/>
+        <c:axId val="50030001"/>
+        <c:axId val="50030002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50020001"/>
+        <c:axId val="50030001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="50020002"/>
+        <c:crossAx val="50030002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50020002"/>
+        <c:axId val="50030002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2546,7 +2706,7 @@
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50020001"/>
+        <c:crossAx val="50030001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2565,7 +2725,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:style val="10"/>
@@ -2685,24 +2845,24 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50030001"/>
-        <c:axId val="50030002"/>
+        <c:axId val="50040001"/>
+        <c:axId val="50040002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50030001"/>
+        <c:axId val="50040001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="50030002"/>
+        <c:crossAx val="50040002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50030002"/>
+        <c:axId val="50040002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2728,7 +2888,7 @@
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50030001"/>
+        <c:crossAx val="50040001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2747,7 +2907,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:style val="10"/>
@@ -2867,24 +3027,24 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50040001"/>
-        <c:axId val="50040002"/>
+        <c:axId val="50050001"/>
+        <c:axId val="50050002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50040001"/>
+        <c:axId val="50050001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="50040002"/>
+        <c:crossAx val="50050002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50040002"/>
+        <c:axId val="50050002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2910,7 +3070,7 @@
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50040001"/>
+        <c:crossAx val="50050001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2929,7 +3089,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:style val="10"/>
@@ -3049,24 +3209,24 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50050001"/>
-        <c:axId val="50050002"/>
+        <c:axId val="50060001"/>
+        <c:axId val="50060002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50050001"/>
+        <c:axId val="50060001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="50050002"/>
+        <c:crossAx val="50060002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50050002"/>
+        <c:axId val="50060002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3092,7 +3252,7 @@
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50050001"/>
+        <c:crossAx val="50060001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3111,7 +3271,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:style val="10"/>
@@ -3255,24 +3415,24 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50060001"/>
-        <c:axId val="50060002"/>
+        <c:axId val="50070001"/>
+        <c:axId val="50070002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50060001"/>
+        <c:axId val="50070001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="50060002"/>
+        <c:crossAx val="50070002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50060002"/>
+        <c:axId val="50070002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3298,7 +3458,7 @@
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50060001"/>
+        <c:crossAx val="50070001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3321,15 +3481,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1371600</xdr:colOff>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3351,15 +3511,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1371600</xdr:colOff>
+      <xdr:row>68</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3381,15 +3541,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>35</xdr:row>
+      <xdr:row>68</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3411,15 +3571,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>69</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>35</xdr:row>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1371600</xdr:colOff>
+      <xdr:row>85</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3441,15 +3601,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>69</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>85</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3471,15 +3631,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>86</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1371600</xdr:colOff>
+      <xdr:row>102</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3494,6 +3654,36 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 7"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -12464,7 +12654,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -12712,11 +12902,11 @@
         <v>522</v>
       </c>
       <c r="B23" s="13">
-        <f>'Memory'!$R$21/1E9</f>
+        <f>('Memory'!$R$21)/1E9</f>
         <v>159.117270492</v>
       </c>
       <c r="C23" s="13">
-        <f>'Memory'!$S$21/1E9</f>
+        <f>('Memory'!$S$21)/1E9</f>
         <v>22.349822332</v>
       </c>
     </row>
@@ -12725,11 +12915,11 @@
         <v>523</v>
       </c>
       <c r="B24" s="13">
-        <f>'Memory'!$P$29/1E9</f>
+        <f>('Memory'!$P$29)/1E9</f>
         <v>7.232045056</v>
       </c>
       <c r="C24" s="13">
-        <f>'Memory'!$Q$29/1E9</f>
+        <f>('Memory'!$Q$29)/1E9</f>
         <v>7.232045056</v>
       </c>
     </row>
@@ -12738,11 +12928,11 @@
         <v>524</v>
       </c>
       <c r="B25" s="13">
-        <f>'Memory'!$R$21+'Memory'!$P$29/1E9</f>
+        <f>('Memory'!$R$21+'Memory'!$P$29)/1E9</f>
         <v>166.349315548</v>
       </c>
       <c r="C25" s="13">
-        <f>'Memory'!$S$21+'Memory'!$Q$29/1E9</f>
+        <f>('Memory'!$S$21+'Memory'!$Q$29)/1E9</f>
         <v>29.581867388</v>
       </c>
     </row>
@@ -12751,11 +12941,11 @@
         <v>525</v>
       </c>
       <c r="B26" s="13">
-        <f>'Memory'!$P$33/1E9</f>
+        <f>('Memory'!$P$33)/1E9</f>
         <v>7.232045056</v>
       </c>
       <c r="C26" s="13">
-        <f>'Memory'!$Q$33/1E9</f>
+        <f>('Memory'!$Q$33)/1E9</f>
         <v>7.232045056</v>
       </c>
     </row>
@@ -12764,12 +12954,56 @@
         <v>526</v>
       </c>
       <c r="B27" s="13">
-        <f>'Memory'!$R$21+'Memory'!$P$33/1E9</f>
+        <f>('Memory'!$R$21+'Memory'!$P$33)/1E9</f>
         <v>166.349315548</v>
       </c>
       <c r="C27" s="13">
-        <f>'Memory'!$S$21+'Memory'!$Q$33/1E9</f>
+        <f>('Memory'!$S$21+'Memory'!$Q$33)/1E9</f>
         <v>29.581867388</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="B31" s="13">
+        <f>'Prefill_8K'!$AE$23</f>
+        <v>228.384427393024</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="B32" s="13">
+        <f>'Prefill_8K'!$AF$23</f>
+        <v>55.63931418624</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="B33" s="13">
+        <f>'Decode_1M'!$AE$23</f>
+        <v>14.0354134102</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="B34" s="13">
+        <f>'Decode_1M'!$AF$23</f>
+        <v>2.3548076118</v>
       </c>
     </row>
   </sheetData>
@@ -12789,47 +13023,47 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="3" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="4" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="4" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="4" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="4" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -12837,55 +13071,55 @@
         <v>67</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="4" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="4" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="4" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="4" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -12893,15 +13127,15 @@
         <v>460</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
     </row>
   </sheetData>
@@ -12922,17 +13156,17 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="7" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -12942,16 +13176,16 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>460</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>460</v>
@@ -12962,7 +13196,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="4" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="B6" s="12">
         <f>IF(ABS(G6)&gt;=1E15,G6/1E15,IF(ABS(G6)&gt;=1E12,G6/1E12,IF(ABS(G6)&gt;=1E9,G6/1E9,IF(ABS(G6)&gt;=1E6,G6/1E6,G6))))</f>
@@ -12981,7 +13215,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="G6" s="13">
         <f>'Prefill_8K'!$AE$13</f>
@@ -12994,7 +13228,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="4" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="B7" s="12">
         <f>IF(ABS(G7)&gt;=1E15,G7/1E15,IF(ABS(G7)&gt;=1E12,G7/1E12,IF(ABS(G7)&gt;=1E9,G7/1E9,IF(ABS(G7)&gt;=1E6,G7/1E6,G7))))</f>
@@ -13013,7 +13247,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="G7" s="13">
         <f>'Prefill_8K'!$AE$14</f>
@@ -13026,7 +13260,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="4" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B8" s="12">
         <f>IF(ABS(G8)&gt;=1E15,G8/1E15,IF(ABS(G8)&gt;=1E12,G8/1E12,IF(ABS(G8)&gt;=1E9,G8/1E9,IF(ABS(G8)&gt;=1E6,G8/1E6,G8))))</f>
@@ -13045,7 +13279,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="G8" s="13">
         <f>'Prefill_8K'!$AE$15</f>
@@ -13058,7 +13292,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="14" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="B9" s="14">
         <f>IF(ABS(G9)&gt;=1E15,G9/1E15,IF(ABS(G9)&gt;=1E12,G9/1E12,IF(ABS(G9)&gt;=1E9,G9/1E9,IF(ABS(G9)&gt;=1E6,G9/1E6,G9))))</f>
@@ -13077,7 +13311,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="G9" s="13">
         <f>'Prefill_8K'!$AE$16</f>
@@ -13090,7 +13324,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="4" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="B10" s="12">
         <f>IF(ABS(G10)&gt;=1E12,G10/1E12,IF(ABS(G10)&gt;=1E9,G10/1E9,IF(ABS(G10)&gt;=1E6,G10/1E6,IF(ABS(G10)&gt;=1E3,G10/1E3,G10))))</f>
@@ -13109,7 +13343,7 @@
         <v>GB</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="G10" s="13">
         <f>'Prefill_8K'!$AE$17</f>
@@ -13122,7 +13356,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="4" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="B11" s="12">
         <f>IF(ABS(G11)&gt;=1E12,G11/1E12,IF(ABS(G11)&gt;=1E9,G11/1E9,IF(ABS(G11)&gt;=1E6,G11/1E6,IF(ABS(G11)&gt;=1E3,G11/1E3,G11))))</f>
@@ -13141,7 +13375,7 @@
         <v>GB</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="G11" s="13">
         <f>'Prefill_8K'!$AE$18</f>
@@ -13154,7 +13388,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="4" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="B12" s="12">
         <f>IF(ABS(G12)&gt;=1E12,G12/1E12,IF(ABS(G12)&gt;=1E9,G12/1E9,IF(ABS(G12)&gt;=1E6,G12/1E6,IF(ABS(G12)&gt;=1E3,G12/1E3,G12))))</f>
@@ -13173,7 +13407,7 @@
         <v>GB</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="G12" s="13">
         <f>'Prefill_8K'!$AE$19</f>
@@ -13186,7 +13420,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="14" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="B13" s="14">
         <f>IF(ABS(G13)&gt;=1E12,G13/1E12,IF(ABS(G13)&gt;=1E9,G13/1E9,IF(ABS(G13)&gt;=1E6,G13/1E6,IF(ABS(G13)&gt;=1E3,G13/1E3,G13))))</f>
@@ -13205,7 +13439,7 @@
         <v>GB</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="G13" s="13">
         <f>'Prefill_8K'!$AE$20</f>
@@ -13218,7 +13452,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="4" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="B14" s="12">
         <f>G14</f>
@@ -13235,7 +13469,7 @@
         <v>159</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="G14" s="13">
         <f>'Prefill_8K'!$AE$17/(PrefillTargetMs/1000)/1E9</f>
@@ -13248,7 +13482,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="4" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="B15" s="12">
         <f>G15</f>
@@ -13265,7 +13499,7 @@
         <v>159</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="G15" s="13">
         <f>'Prefill_8K'!$AE$18/(PrefillTargetMs/1000)/1E9</f>
@@ -13278,7 +13512,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="4" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="B16" s="12">
         <f>G16</f>
@@ -13295,7 +13529,7 @@
         <v>159</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="G16" s="13">
         <f>'Prefill_8K'!$AE$19/(PrefillTargetMs/1000)/1E9</f>
@@ -13308,7 +13542,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="4" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="B17" s="12">
         <f>G17</f>
@@ -13325,7 +13559,7 @@
         <v>155</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="G17" s="13">
         <f>'Prefill_8K'!$AE$23</f>
@@ -13338,7 +13572,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="4" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="B18" s="12">
         <f>IF(ABS(G18)&gt;=1E12,G18/1E12,IF(ABS(G18)&gt;=1E9,G18/1E9,IF(ABS(G18)&gt;=1E6,G18/1E6,IF(ABS(G18)&gt;=1E3,G18/1E3,G18))))</f>
@@ -13357,7 +13591,7 @@
         <v>B</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="G18" s="13">
         <f>'Prefill_8K'!$AE$21</f>
@@ -13370,7 +13604,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="4" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="B19" s="12">
         <f>G19</f>
@@ -13387,7 +13621,7 @@
         <v>159</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="G19" s="13">
         <f>'Prefill_8K'!$AE$21/(PrefillTargetMs/1000)/1E9</f>
@@ -13400,7 +13634,7 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="4" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="B20" s="12">
         <f>IF(ABS(G20)&gt;=1E12,G20/1E12,IF(ABS(G20)&gt;=1E9,G20/1E9,IF(ABS(G20)&gt;=1E6,G20/1E6,IF(ABS(G20)&gt;=1E3,G20/1E3,G20))))</f>
@@ -13419,7 +13653,7 @@
         <v>G params</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="G20" s="13">
         <f>'Memory'!$P$18</f>
@@ -13432,7 +13666,7 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="4" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="B21" s="12">
         <f>IF(ABS(G21)&gt;=1E12,G21/1E12,IF(ABS(G21)&gt;=1E9,G21/1E9,IF(ABS(G21)&gt;=1E6,G21/1E6,IF(ABS(G21)&gt;=1E3,G21/1E3,G21))))</f>
@@ -13451,7 +13685,7 @@
         <v>G params</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="G21" s="13">
         <f>'Memory'!$P$19</f>
@@ -13464,7 +13698,7 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="4" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="B22" s="12">
         <f>IF(ABS(G22)&gt;=1E12,G22/1E12,IF(ABS(G22)&gt;=1E9,G22/1E9,IF(ABS(G22)&gt;=1E6,G22/1E6,IF(ABS(G22)&gt;=1E3,G22/1E3,G22))))</f>
@@ -13483,7 +13717,7 @@
         <v>G params</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="G22" s="13">
         <f>'Memory'!$P$20</f>
@@ -13496,7 +13730,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="14" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="B23" s="14">
         <f>IF(ABS(G23)&gt;=1E12,G23/1E12,IF(ABS(G23)&gt;=1E9,G23/1E9,IF(ABS(G23)&gt;=1E6,G23/1E6,IF(ABS(G23)&gt;=1E3,G23/1E3,G23))))</f>
@@ -13515,7 +13749,7 @@
         <v>G params</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="G23" s="13">
         <f>'Memory'!$P$21</f>
@@ -13528,7 +13762,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="4" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="B24" s="12">
         <f>IF(ABS(G24)&gt;=1E12,G24/1E12,IF(ABS(G24)&gt;=1E9,G24/1E9,IF(ABS(G24)&gt;=1E6,G24/1E6,IF(ABS(G24)&gt;=1E3,G24/1E3,G24))))</f>
@@ -13547,7 +13781,7 @@
         <v>GB</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="G24" s="13">
         <f>'Memory'!$R$18</f>
@@ -13560,7 +13794,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="4" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="B25" s="12">
         <f>IF(ABS(G25)&gt;=1E12,G25/1E12,IF(ABS(G25)&gt;=1E9,G25/1E9,IF(ABS(G25)&gt;=1E6,G25/1E6,IF(ABS(G25)&gt;=1E3,G25/1E3,G25))))</f>
@@ -13579,7 +13813,7 @@
         <v>GB</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="G25" s="13">
         <f>'Memory'!$R$19</f>
@@ -13592,7 +13826,7 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="4" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="B26" s="12">
         <f>IF(ABS(G26)&gt;=1E12,G26/1E12,IF(ABS(G26)&gt;=1E9,G26/1E9,IF(ABS(G26)&gt;=1E6,G26/1E6,IF(ABS(G26)&gt;=1E3,G26/1E3,G26))))</f>
@@ -13611,7 +13845,7 @@
         <v>GB</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="G26" s="13">
         <f>'Memory'!$R$20</f>
@@ -13624,7 +13858,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="14" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="B27" s="14">
         <f>IF(ABS(G27)&gt;=1E12,G27/1E12,IF(ABS(G27)&gt;=1E9,G27/1E9,IF(ABS(G27)&gt;=1E6,G27/1E6,IF(ABS(G27)&gt;=1E3,G27/1E3,G27))))</f>
@@ -13643,7 +13877,7 @@
         <v>GB</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="G27" s="13">
         <f>'Memory'!$R$21</f>
@@ -13656,7 +13890,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="4" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="B28" s="12">
         <f>IF(ABS(G28)&gt;=1E12,G28/1E12,IF(ABS(G28)&gt;=1E9,G28/1E9,IF(ABS(G28)&gt;=1E6,G28/1E6,IF(ABS(G28)&gt;=1E3,G28/1E3,G28))))</f>
@@ -13675,7 +13909,7 @@
         <v>GB</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="G28" s="13">
         <f>'Memory'!$P$26</f>
@@ -13688,7 +13922,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="4" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="B29" s="12">
         <f>IF(ABS(G29)&gt;=1E12,G29/1E12,IF(ABS(G29)&gt;=1E9,G29/1E9,IF(ABS(G29)&gt;=1E6,G29/1E6,IF(ABS(G29)&gt;=1E3,G29/1E3,G29))))</f>
@@ -13707,7 +13941,7 @@
         <v>GB</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="G29" s="13">
         <f>'Memory'!$P$27</f>
@@ -13720,7 +13954,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="4" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="B30" s="12">
         <f>IF(ABS(G30)&gt;=1E12,G30/1E12,IF(ABS(G30)&gt;=1E9,G30/1E9,IF(ABS(G30)&gt;=1E6,G30/1E6,IF(ABS(G30)&gt;=1E3,G30/1E3,G30))))</f>
@@ -13739,7 +13973,7 @@
         <v>MB</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="G30" s="13">
         <f>'Memory'!$P$28</f>
@@ -13752,7 +13986,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="4" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="B31" s="12">
         <f>IF(ABS(G31)&gt;=1E12,G31/1E12,IF(ABS(G31)&gt;=1E9,G31/1E9,IF(ABS(G31)&gt;=1E6,G31/1E6,IF(ABS(G31)&gt;=1E3,G31/1E3,G31))))</f>
@@ -13771,7 +14005,7 @@
         <v>GB</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="G31" s="13">
         <f>'Memory'!$P$29</f>
@@ -13784,7 +14018,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="14" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="B32" s="14">
         <f>IF(ABS(G32)&gt;=1E12,G32/1E12,IF(ABS(G32)&gt;=1E9,G32/1E9,IF(ABS(G32)&gt;=1E6,G32/1E6,IF(ABS(G32)&gt;=1E3,G32/1E3,G32))))</f>
@@ -13803,7 +14037,7 @@
         <v>GB</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="G32" s="13">
         <f>'Memory'!$R$21+'Memory'!$P$29</f>
@@ -13816,7 +14050,7 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="7" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
@@ -13826,16 +14060,16 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="3" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>460</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>460</v>
@@ -13846,7 +14080,7 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="4" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="B36" s="12">
         <f>IF(ABS(G36)&gt;=1E15,G36/1E15,IF(ABS(G36)&gt;=1E12,G36/1E12,IF(ABS(G36)&gt;=1E9,G36/1E9,IF(ABS(G36)&gt;=1E6,G36/1E6,G36))))</f>
@@ -13865,7 +14099,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="G36" s="13">
         <f>'Prefill_8K'!$AF$13</f>
@@ -13878,7 +14112,7 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="4" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="B37" s="12">
         <f>IF(ABS(G37)&gt;=1E15,G37/1E15,IF(ABS(G37)&gt;=1E12,G37/1E12,IF(ABS(G37)&gt;=1E9,G37/1E9,IF(ABS(G37)&gt;=1E6,G37/1E6,G37))))</f>
@@ -13897,7 +14131,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="G37" s="13">
         <f>'Prefill_8K'!$AF$14</f>
@@ -13910,7 +14144,7 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="4" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B38" s="12">
         <f>IF(ABS(G38)&gt;=1E15,G38/1E15,IF(ABS(G38)&gt;=1E12,G38/1E12,IF(ABS(G38)&gt;=1E9,G38/1E9,IF(ABS(G38)&gt;=1E6,G38/1E6,G38))))</f>
@@ -13929,7 +14163,7 @@
         <v>MFLOPs</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="G38" s="13">
         <f>'Prefill_8K'!$AF$15</f>
@@ -13942,7 +14176,7 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="14" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="B39" s="14">
         <f>IF(ABS(G39)&gt;=1E15,G39/1E15,IF(ABS(G39)&gt;=1E12,G39/1E12,IF(ABS(G39)&gt;=1E9,G39/1E9,IF(ABS(G39)&gt;=1E6,G39/1E6,G39))))</f>
@@ -13961,7 +14195,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="G39" s="13">
         <f>'Prefill_8K'!$AF$16</f>
@@ -13974,7 +14208,7 @@
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="4" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="B40" s="12">
         <f>IF(ABS(G40)&gt;=1E12,G40/1E12,IF(ABS(G40)&gt;=1E9,G40/1E9,IF(ABS(G40)&gt;=1E6,G40/1E6,IF(ABS(G40)&gt;=1E3,G40/1E3,G40))))</f>
@@ -13993,7 +14227,7 @@
         <v>GB</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="G40" s="13">
         <f>'Prefill_8K'!$AF$17</f>
@@ -14006,7 +14240,7 @@
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="4" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="B41" s="12">
         <f>IF(ABS(G41)&gt;=1E12,G41/1E12,IF(ABS(G41)&gt;=1E9,G41/1E9,IF(ABS(G41)&gt;=1E6,G41/1E6,IF(ABS(G41)&gt;=1E3,G41/1E3,G41))))</f>
@@ -14025,7 +14259,7 @@
         <v>GB</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="G41" s="13">
         <f>'Prefill_8K'!$AF$18</f>
@@ -14038,7 +14272,7 @@
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="4" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="B42" s="12">
         <f>IF(ABS(G42)&gt;=1E12,G42/1E12,IF(ABS(G42)&gt;=1E9,G42/1E9,IF(ABS(G42)&gt;=1E6,G42/1E6,IF(ABS(G42)&gt;=1E3,G42/1E3,G42))))</f>
@@ -14057,7 +14291,7 @@
         <v>MB</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="G42" s="13">
         <f>'Prefill_8K'!$AF$19</f>
@@ -14070,7 +14304,7 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="14" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="B43" s="14">
         <f>IF(ABS(G43)&gt;=1E12,G43/1E12,IF(ABS(G43)&gt;=1E9,G43/1E9,IF(ABS(G43)&gt;=1E6,G43/1E6,IF(ABS(G43)&gt;=1E3,G43/1E3,G43))))</f>
@@ -14089,7 +14323,7 @@
         <v>GB</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="G43" s="13">
         <f>'Prefill_8K'!$AF$20</f>
@@ -14102,7 +14336,7 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="4" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="B44" s="12">
         <f>G44</f>
@@ -14119,7 +14353,7 @@
         <v>159</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="G44" s="13">
         <f>'Prefill_8K'!$AF$17/(PrefillTargetMs/1000)/1E9</f>
@@ -14132,7 +14366,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="4" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="B45" s="12">
         <f>G45</f>
@@ -14149,7 +14383,7 @@
         <v>159</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="G45" s="13">
         <f>'Prefill_8K'!$AF$18/(PrefillTargetMs/1000)/1E9</f>
@@ -14162,7 +14396,7 @@
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="4" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="B46" s="12">
         <f>G46</f>
@@ -14179,7 +14413,7 @@
         <v>159</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="G46" s="13">
         <f>'Prefill_8K'!$AF$19/(PrefillTargetMs/1000)/1E9</f>
@@ -14192,7 +14426,7 @@
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="4" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="B47" s="12">
         <f>G47</f>
@@ -14209,7 +14443,7 @@
         <v>155</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="G47" s="13">
         <f>'Prefill_8K'!$AF$23</f>
@@ -14222,7 +14456,7 @@
     </row>
     <row r="48" spans="1:8">
       <c r="A48" s="4" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="B48" s="12">
         <f>IF(ABS(G48)&gt;=1E12,G48/1E12,IF(ABS(G48)&gt;=1E9,G48/1E9,IF(ABS(G48)&gt;=1E6,G48/1E6,IF(ABS(G48)&gt;=1E3,G48/1E3,G48))))</f>
@@ -14241,7 +14475,7 @@
         <v>MB</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="G48" s="13">
         <f>'Prefill_8K'!$AF$21</f>
@@ -14254,7 +14488,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="4" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="B49" s="12">
         <f>G49</f>
@@ -14271,7 +14505,7 @@
         <v>159</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="G49" s="13">
         <f>'Prefill_8K'!$AF$21/(PrefillTargetMs/1000)/1E9</f>
@@ -14284,7 +14518,7 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="4" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="B50" s="12">
         <f>IF(ABS(G50)&gt;=1E12,G50/1E12,IF(ABS(G50)&gt;=1E9,G50/1E9,IF(ABS(G50)&gt;=1E6,G50/1E6,IF(ABS(G50)&gt;=1E3,G50/1E3,G50))))</f>
@@ -14303,7 +14537,7 @@
         <v>G params</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="G50" s="13">
         <f>'Memory'!$Q$18</f>
@@ -14316,7 +14550,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="4" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="B51" s="12">
         <f>IF(ABS(G51)&gt;=1E12,G51/1E12,IF(ABS(G51)&gt;=1E9,G51/1E9,IF(ABS(G51)&gt;=1E6,G51/1E6,IF(ABS(G51)&gt;=1E3,G51/1E3,G51))))</f>
@@ -14335,7 +14569,7 @@
         <v>G params</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="G51" s="13">
         <f>'Memory'!$Q$19</f>
@@ -14348,7 +14582,7 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="4" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="B52" s="12">
         <f>IF(ABS(G52)&gt;=1E12,G52/1E12,IF(ABS(G52)&gt;=1E9,G52/1E9,IF(ABS(G52)&gt;=1E6,G52/1E6,IF(ABS(G52)&gt;=1E3,G52/1E3,G52))))</f>
@@ -14367,7 +14601,7 @@
         <v>M params</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="G52" s="13">
         <f>'Memory'!$Q$20</f>
@@ -14380,7 +14614,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="14" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="B53" s="14">
         <f>IF(ABS(G53)&gt;=1E12,G53/1E12,IF(ABS(G53)&gt;=1E9,G53/1E9,IF(ABS(G53)&gt;=1E6,G53/1E6,IF(ABS(G53)&gt;=1E3,G53/1E3,G53))))</f>
@@ -14399,7 +14633,7 @@
         <v>G params</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="G53" s="13">
         <f>'Memory'!$Q$21</f>
@@ -14412,7 +14646,7 @@
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="4" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="B54" s="12">
         <f>IF(ABS(G54)&gt;=1E12,G54/1E12,IF(ABS(G54)&gt;=1E9,G54/1E9,IF(ABS(G54)&gt;=1E6,G54/1E6,IF(ABS(G54)&gt;=1E3,G54/1E3,G54))))</f>
@@ -14431,7 +14665,7 @@
         <v>GB</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="G54" s="13">
         <f>'Memory'!$S$18</f>
@@ -14444,7 +14678,7 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="4" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="B55" s="12">
         <f>IF(ABS(G55)&gt;=1E12,G55/1E12,IF(ABS(G55)&gt;=1E9,G55/1E9,IF(ABS(G55)&gt;=1E6,G55/1E6,IF(ABS(G55)&gt;=1E3,G55/1E3,G55))))</f>
@@ -14463,7 +14697,7 @@
         <v>GB</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="G55" s="13">
         <f>'Memory'!$S$19</f>
@@ -14476,7 +14710,7 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="4" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="B56" s="12">
         <f>IF(ABS(G56)&gt;=1E12,G56/1E12,IF(ABS(G56)&gt;=1E9,G56/1E9,IF(ABS(G56)&gt;=1E6,G56/1E6,IF(ABS(G56)&gt;=1E3,G56/1E3,G56))))</f>
@@ -14495,7 +14729,7 @@
         <v>MB</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="G56" s="13">
         <f>'Memory'!$S$20</f>
@@ -14508,7 +14742,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="14" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="B57" s="14">
         <f>IF(ABS(G57)&gt;=1E12,G57/1E12,IF(ABS(G57)&gt;=1E9,G57/1E9,IF(ABS(G57)&gt;=1E6,G57/1E6,IF(ABS(G57)&gt;=1E3,G57/1E3,G57))))</f>
@@ -14527,7 +14761,7 @@
         <v>GB</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="G57" s="13">
         <f>'Memory'!$S$21</f>
@@ -14540,7 +14774,7 @@
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="4" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="B58" s="12">
         <f>IF(ABS(G58)&gt;=1E12,G58/1E12,IF(ABS(G58)&gt;=1E9,G58/1E9,IF(ABS(G58)&gt;=1E6,G58/1E6,IF(ABS(G58)&gt;=1E3,G58/1E3,G58))))</f>
@@ -14559,7 +14793,7 @@
         <v>GB</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="G58" s="13">
         <f>'Memory'!$Q$26</f>
@@ -14572,7 +14806,7 @@
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="4" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="B59" s="12">
         <f>IF(ABS(G59)&gt;=1E12,G59/1E12,IF(ABS(G59)&gt;=1E9,G59/1E9,IF(ABS(G59)&gt;=1E6,G59/1E6,IF(ABS(G59)&gt;=1E3,G59/1E3,G59))))</f>
@@ -14591,7 +14825,7 @@
         <v>GB</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="G59" s="13">
         <f>'Memory'!$Q$27</f>
@@ -14604,7 +14838,7 @@
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="4" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="B60" s="12">
         <f>IF(ABS(G60)&gt;=1E12,G60/1E12,IF(ABS(G60)&gt;=1E9,G60/1E9,IF(ABS(G60)&gt;=1E6,G60/1E6,IF(ABS(G60)&gt;=1E3,G60/1E3,G60))))</f>
@@ -14623,7 +14857,7 @@
         <v>MB</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="G60" s="13">
         <f>'Memory'!$Q$28</f>
@@ -14636,7 +14870,7 @@
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="4" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="B61" s="12">
         <f>IF(ABS(G61)&gt;=1E12,G61/1E12,IF(ABS(G61)&gt;=1E9,G61/1E9,IF(ABS(G61)&gt;=1E6,G61/1E6,IF(ABS(G61)&gt;=1E3,G61/1E3,G61))))</f>
@@ -14655,7 +14889,7 @@
         <v>GB</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="G61" s="13">
         <f>'Memory'!$Q$29</f>
@@ -14668,7 +14902,7 @@
     </row>
     <row r="62" spans="1:8">
       <c r="A62" s="14" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="B62" s="14">
         <f>IF(ABS(G62)&gt;=1E12,G62/1E12,IF(ABS(G62)&gt;=1E9,G62/1E9,IF(ABS(G62)&gt;=1E6,G62/1E6,IF(ABS(G62)&gt;=1E3,G62/1E3,G62))))</f>
@@ -14687,7 +14921,7 @@
         <v>GB</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="G62" s="13">
         <f>'Memory'!$S$21+'Memory'!$Q$29</f>

</xml_diff>

<commit_message>
Clarify resident capacity comparison
</commit_message>
<xml_diff>
--- a/calculate/deepseek_v4_flash_calculator.xlsx
+++ b/calculate/deepseek_v4_flash_calculator.xlsx
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="609">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="607">
   <si>
     <t>DeepSeek V4 Flash - Editable Architecture Parameters</t>
   </si>
@@ -1765,22 +1765,16 @@
     <t>说明：参数容量只由模型结构、dtype 和 TP 分片决定，与 Prefill/Decode 场景无关；两列分别是单 Rank 值，不相加。</t>
   </si>
   <si>
-    <t>推理场景容量项</t>
+    <t>单 Rank 容量项</t>
   </si>
   <si>
     <t>静态参数（场景共用）</t>
   </si>
   <si>
-    <t>Prefill 预分配 KV+State</t>
-  </si>
-  <si>
-    <t>Prefill 总驻留（参数+KV）</t>
-  </si>
-  <si>
-    <t>Decode 预分配 KV+State</t>
-  </si>
-  <si>
-    <t>Decode 总驻留（参数+KV）</t>
+    <t>预分配 KV+State（Prefill/Decode 当前相同）</t>
+  </si>
+  <si>
+    <t>总驻留（静态参数+KV+State）</t>
   </si>
   <si>
     <t>算力需求场景</t>
@@ -3287,7 +3281,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Prefill / Decode 单 Rank 容量（TP 配置独立）</a:t>
+              <a:t>TP1 vs TP8：单 Rank 推理驻留容量</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -3311,33 +3305,27 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Comparison!$A$23:$A$27</c:f>
+              <c:f>Comparison!$A$23:$A$25</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>静态参数（场景共用）</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Prefill 预分配 KV+State</c:v>
+                  <c:v>预分配 KV+State（Prefill/Decode 当前相同）</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Prefill 总驻留（参数+KV）</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Decode 预分配 KV+State</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Decode 总驻留（参数+KV）</c:v>
+                  <c:v>总驻留（静态参数+KV+State）</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Comparison!$B$23:$B$27</c:f>
+              <c:f>Comparison!$B$23:$B$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>159.117270492</c:v>
                 </c:pt>
@@ -3345,12 +3333,6 @@
                   <c:v>7.232045056</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>166.349315548</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>7.232045056</c:v>
-                </c:pt>
-                <c:pt idx="4">
                   <c:v>166.349315548</c:v>
                 </c:pt>
               </c:numCache>
@@ -3369,33 +3351,27 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Comparison!$A$23:$A$27</c:f>
+              <c:f>Comparison!$A$23:$A$25</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>静态参数（场景共用）</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Prefill 预分配 KV+State</c:v>
+                  <c:v>预分配 KV+State（Prefill/Decode 当前相同）</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Prefill 总驻留（参数+KV）</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Decode 预分配 KV+State</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Decode 总驻留（参数+KV）</c:v>
+                  <c:v>总驻留（静态参数+KV+State）</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Comparison!$C$23:$C$27</c:f>
+              <c:f>Comparison!$C$23:$C$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>22.349822332</c:v>
                 </c:pt>
@@ -3403,12 +3379,6 @@
                   <c:v>7.232045056</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>29.581867388</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>7.232045056</c:v>
-                </c:pt>
-                <c:pt idx="4">
                   <c:v>29.581867388</c:v>
                 </c:pt>
               </c:numCache>
@@ -12936,43 +12906,17 @@
         <v>29.581867388</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="4" t="s">
-        <v>525</v>
-      </c>
-      <c r="B26" s="13">
-        <f>('Memory'!$P$33)/1E9</f>
-        <v>7.232045056</v>
-      </c>
-      <c r="C26" s="13">
-        <f>('Memory'!$Q$33)/1E9</f>
-        <v>7.232045056</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" s="4" t="s">
-        <v>526</v>
-      </c>
-      <c r="B27" s="13">
-        <f>('Memory'!$R$21+'Memory'!$P$33)/1E9</f>
-        <v>166.349315548</v>
-      </c>
-      <c r="C27" s="13">
-        <f>('Memory'!$S$21+'Memory'!$Q$33)/1E9</f>
-        <v>29.581867388</v>
-      </c>
-    </row>
     <row r="30" spans="1:3">
       <c r="A30" s="3" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="4" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="B31" s="13">
         <f>'Prefill_8K'!$AE$23</f>
@@ -12981,7 +12925,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="4" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="B32" s="13">
         <f>'Prefill_8K'!$AF$23</f>
@@ -12990,7 +12934,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="4" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="B33" s="13">
         <f>'Decode_1M'!$AE$23</f>
@@ -12999,7 +12943,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="4" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="B34" s="13">
         <f>'Decode_1M'!$AF$23</f>
@@ -13023,47 +12967,47 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="3" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="4" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="4" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="4" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="4" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -13071,55 +13015,55 @@
         <v>67</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="4" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="4" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="4" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -13127,15 +13071,15 @@
         <v>460</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
   </sheetData>
@@ -13156,17 +13100,17 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="7" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -13176,16 +13120,16 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>460</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>460</v>
@@ -13196,7 +13140,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="4" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="B6" s="12">
         <f>IF(ABS(G6)&gt;=1E15,G6/1E15,IF(ABS(G6)&gt;=1E12,G6/1E12,IF(ABS(G6)&gt;=1E9,G6/1E9,IF(ABS(G6)&gt;=1E6,G6/1E6,G6))))</f>
@@ -13215,7 +13159,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="G6" s="13">
         <f>'Prefill_8K'!$AE$13</f>
@@ -13228,7 +13172,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="4" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="B7" s="12">
         <f>IF(ABS(G7)&gt;=1E15,G7/1E15,IF(ABS(G7)&gt;=1E12,G7/1E12,IF(ABS(G7)&gt;=1E9,G7/1E9,IF(ABS(G7)&gt;=1E6,G7/1E6,G7))))</f>
@@ -13247,7 +13191,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="G7" s="13">
         <f>'Prefill_8K'!$AE$14</f>
@@ -13260,7 +13204,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="4" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="B8" s="12">
         <f>IF(ABS(G8)&gt;=1E15,G8/1E15,IF(ABS(G8)&gt;=1E12,G8/1E12,IF(ABS(G8)&gt;=1E9,G8/1E9,IF(ABS(G8)&gt;=1E6,G8/1E6,G8))))</f>
@@ -13279,7 +13223,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="G8" s="13">
         <f>'Prefill_8K'!$AE$15</f>
@@ -13292,7 +13236,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="14" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="B9" s="14">
         <f>IF(ABS(G9)&gt;=1E15,G9/1E15,IF(ABS(G9)&gt;=1E12,G9/1E12,IF(ABS(G9)&gt;=1E9,G9/1E9,IF(ABS(G9)&gt;=1E6,G9/1E6,G9))))</f>
@@ -13311,7 +13255,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="G9" s="13">
         <f>'Prefill_8K'!$AE$16</f>
@@ -13324,7 +13268,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="4" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="B10" s="12">
         <f>IF(ABS(G10)&gt;=1E12,G10/1E12,IF(ABS(G10)&gt;=1E9,G10/1E9,IF(ABS(G10)&gt;=1E6,G10/1E6,IF(ABS(G10)&gt;=1E3,G10/1E3,G10))))</f>
@@ -13343,7 +13287,7 @@
         <v>GB</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="G10" s="13">
         <f>'Prefill_8K'!$AE$17</f>
@@ -13356,7 +13300,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="4" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="B11" s="12">
         <f>IF(ABS(G11)&gt;=1E12,G11/1E12,IF(ABS(G11)&gt;=1E9,G11/1E9,IF(ABS(G11)&gt;=1E6,G11/1E6,IF(ABS(G11)&gt;=1E3,G11/1E3,G11))))</f>
@@ -13375,7 +13319,7 @@
         <v>GB</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="G11" s="13">
         <f>'Prefill_8K'!$AE$18</f>
@@ -13388,7 +13332,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="4" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B12" s="12">
         <f>IF(ABS(G12)&gt;=1E12,G12/1E12,IF(ABS(G12)&gt;=1E9,G12/1E9,IF(ABS(G12)&gt;=1E6,G12/1E6,IF(ABS(G12)&gt;=1E3,G12/1E3,G12))))</f>
@@ -13407,7 +13351,7 @@
         <v>GB</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="G12" s="13">
         <f>'Prefill_8K'!$AE$19</f>
@@ -13420,7 +13364,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="14" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="B13" s="14">
         <f>IF(ABS(G13)&gt;=1E12,G13/1E12,IF(ABS(G13)&gt;=1E9,G13/1E9,IF(ABS(G13)&gt;=1E6,G13/1E6,IF(ABS(G13)&gt;=1E3,G13/1E3,G13))))</f>
@@ -13439,7 +13383,7 @@
         <v>GB</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="G13" s="13">
         <f>'Prefill_8K'!$AE$20</f>
@@ -13452,7 +13396,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="4" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B14" s="12">
         <f>G14</f>
@@ -13469,7 +13413,7 @@
         <v>159</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="G14" s="13">
         <f>'Prefill_8K'!$AE$17/(PrefillTargetMs/1000)/1E9</f>
@@ -13482,7 +13426,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B15" s="12">
         <f>G15</f>
@@ -13499,7 +13443,7 @@
         <v>159</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="G15" s="13">
         <f>'Prefill_8K'!$AE$18/(PrefillTargetMs/1000)/1E9</f>
@@ -13512,7 +13456,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="4" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="B16" s="12">
         <f>G16</f>
@@ -13529,7 +13473,7 @@
         <v>159</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="G16" s="13">
         <f>'Prefill_8K'!$AE$19/(PrefillTargetMs/1000)/1E9</f>
@@ -13542,7 +13486,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B17" s="12">
         <f>G17</f>
@@ -13559,7 +13503,7 @@
         <v>155</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="G17" s="13">
         <f>'Prefill_8K'!$AE$23</f>
@@ -13572,7 +13516,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B18" s="12">
         <f>IF(ABS(G18)&gt;=1E12,G18/1E12,IF(ABS(G18)&gt;=1E9,G18/1E9,IF(ABS(G18)&gt;=1E6,G18/1E6,IF(ABS(G18)&gt;=1E3,G18/1E3,G18))))</f>
@@ -13591,7 +13535,7 @@
         <v>B</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="G18" s="13">
         <f>'Prefill_8K'!$AE$21</f>
@@ -13604,7 +13548,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="4" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B19" s="12">
         <f>G19</f>
@@ -13621,7 +13565,7 @@
         <v>159</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="G19" s="13">
         <f>'Prefill_8K'!$AE$21/(PrefillTargetMs/1000)/1E9</f>
@@ -13634,7 +13578,7 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="4" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B20" s="12">
         <f>IF(ABS(G20)&gt;=1E12,G20/1E12,IF(ABS(G20)&gt;=1E9,G20/1E9,IF(ABS(G20)&gt;=1E6,G20/1E6,IF(ABS(G20)&gt;=1E3,G20/1E3,G20))))</f>
@@ -13653,7 +13597,7 @@
         <v>G params</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="G20" s="13">
         <f>'Memory'!$P$18</f>
@@ -13666,7 +13610,7 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="4" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B21" s="12">
         <f>IF(ABS(G21)&gt;=1E12,G21/1E12,IF(ABS(G21)&gt;=1E9,G21/1E9,IF(ABS(G21)&gt;=1E6,G21/1E6,IF(ABS(G21)&gt;=1E3,G21/1E3,G21))))</f>
@@ -13685,7 +13629,7 @@
         <v>G params</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="G21" s="13">
         <f>'Memory'!$P$19</f>
@@ -13698,7 +13642,7 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="4" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B22" s="12">
         <f>IF(ABS(G22)&gt;=1E12,G22/1E12,IF(ABS(G22)&gt;=1E9,G22/1E9,IF(ABS(G22)&gt;=1E6,G22/1E6,IF(ABS(G22)&gt;=1E3,G22/1E3,G22))))</f>
@@ -13717,7 +13661,7 @@
         <v>G params</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="G22" s="13">
         <f>'Memory'!$P$20</f>
@@ -13730,7 +13674,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="14" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="B23" s="14">
         <f>IF(ABS(G23)&gt;=1E12,G23/1E12,IF(ABS(G23)&gt;=1E9,G23/1E9,IF(ABS(G23)&gt;=1E6,G23/1E6,IF(ABS(G23)&gt;=1E3,G23/1E3,G23))))</f>
@@ -13749,7 +13693,7 @@
         <v>G params</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="G23" s="13">
         <f>'Memory'!$P$21</f>
@@ -13762,7 +13706,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="4" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="B24" s="12">
         <f>IF(ABS(G24)&gt;=1E12,G24/1E12,IF(ABS(G24)&gt;=1E9,G24/1E9,IF(ABS(G24)&gt;=1E6,G24/1E6,IF(ABS(G24)&gt;=1E3,G24/1E3,G24))))</f>
@@ -13781,7 +13725,7 @@
         <v>GB</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="G24" s="13">
         <f>'Memory'!$R$18</f>
@@ -13794,7 +13738,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="4" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="B25" s="12">
         <f>IF(ABS(G25)&gt;=1E12,G25/1E12,IF(ABS(G25)&gt;=1E9,G25/1E9,IF(ABS(G25)&gt;=1E6,G25/1E6,IF(ABS(G25)&gt;=1E3,G25/1E3,G25))))</f>
@@ -13813,7 +13757,7 @@
         <v>GB</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="G25" s="13">
         <f>'Memory'!$R$19</f>
@@ -13826,7 +13770,7 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="4" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="B26" s="12">
         <f>IF(ABS(G26)&gt;=1E12,G26/1E12,IF(ABS(G26)&gt;=1E9,G26/1E9,IF(ABS(G26)&gt;=1E6,G26/1E6,IF(ABS(G26)&gt;=1E3,G26/1E3,G26))))</f>
@@ -13845,7 +13789,7 @@
         <v>GB</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="G26" s="13">
         <f>'Memory'!$R$20</f>
@@ -13858,7 +13802,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="14" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="B27" s="14">
         <f>IF(ABS(G27)&gt;=1E12,G27/1E12,IF(ABS(G27)&gt;=1E9,G27/1E9,IF(ABS(G27)&gt;=1E6,G27/1E6,IF(ABS(G27)&gt;=1E3,G27/1E3,G27))))</f>
@@ -13877,7 +13821,7 @@
         <v>GB</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G27" s="13">
         <f>'Memory'!$R$21</f>
@@ -13890,7 +13834,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="4" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B28" s="12">
         <f>IF(ABS(G28)&gt;=1E12,G28/1E12,IF(ABS(G28)&gt;=1E9,G28/1E9,IF(ABS(G28)&gt;=1E6,G28/1E6,IF(ABS(G28)&gt;=1E3,G28/1E3,G28))))</f>
@@ -13909,7 +13853,7 @@
         <v>GB</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G28" s="13">
         <f>'Memory'!$P$26</f>
@@ -13922,7 +13866,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="4" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B29" s="12">
         <f>IF(ABS(G29)&gt;=1E12,G29/1E12,IF(ABS(G29)&gt;=1E9,G29/1E9,IF(ABS(G29)&gt;=1E6,G29/1E6,IF(ABS(G29)&gt;=1E3,G29/1E3,G29))))</f>
@@ -13941,7 +13885,7 @@
         <v>GB</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G29" s="13">
         <f>'Memory'!$P$27</f>
@@ -13954,7 +13898,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="4" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B30" s="12">
         <f>IF(ABS(G30)&gt;=1E12,G30/1E12,IF(ABS(G30)&gt;=1E9,G30/1E9,IF(ABS(G30)&gt;=1E6,G30/1E6,IF(ABS(G30)&gt;=1E3,G30/1E3,G30))))</f>
@@ -13973,7 +13917,7 @@
         <v>MB</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G30" s="13">
         <f>'Memory'!$P$28</f>
@@ -13986,7 +13930,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="4" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B31" s="12">
         <f>IF(ABS(G31)&gt;=1E12,G31/1E12,IF(ABS(G31)&gt;=1E9,G31/1E9,IF(ABS(G31)&gt;=1E6,G31/1E6,IF(ABS(G31)&gt;=1E3,G31/1E3,G31))))</f>
@@ -14005,7 +13949,7 @@
         <v>GB</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G31" s="13">
         <f>'Memory'!$P$29</f>
@@ -14018,7 +13962,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="14" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B32" s="14">
         <f>IF(ABS(G32)&gt;=1E12,G32/1E12,IF(ABS(G32)&gt;=1E9,G32/1E9,IF(ABS(G32)&gt;=1E6,G32/1E6,IF(ABS(G32)&gt;=1E3,G32/1E3,G32))))</f>
@@ -14037,7 +13981,7 @@
         <v>GB</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="G32" s="13">
         <f>'Memory'!$R$21+'Memory'!$P$29</f>
@@ -14050,7 +13994,7 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="7" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
@@ -14060,16 +14004,16 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="3" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>460</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>460</v>
@@ -14080,7 +14024,7 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="4" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="B36" s="12">
         <f>IF(ABS(G36)&gt;=1E15,G36/1E15,IF(ABS(G36)&gt;=1E12,G36/1E12,IF(ABS(G36)&gt;=1E9,G36/1E9,IF(ABS(G36)&gt;=1E6,G36/1E6,G36))))</f>
@@ -14099,7 +14043,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="G36" s="13">
         <f>'Prefill_8K'!$AF$13</f>
@@ -14112,7 +14056,7 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="4" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="B37" s="12">
         <f>IF(ABS(G37)&gt;=1E15,G37/1E15,IF(ABS(G37)&gt;=1E12,G37/1E12,IF(ABS(G37)&gt;=1E9,G37/1E9,IF(ABS(G37)&gt;=1E6,G37/1E6,G37))))</f>
@@ -14131,7 +14075,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="G37" s="13">
         <f>'Prefill_8K'!$AF$14</f>
@@ -14144,7 +14088,7 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="4" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="B38" s="12">
         <f>IF(ABS(G38)&gt;=1E15,G38/1E15,IF(ABS(G38)&gt;=1E12,G38/1E12,IF(ABS(G38)&gt;=1E9,G38/1E9,IF(ABS(G38)&gt;=1E6,G38/1E6,G38))))</f>
@@ -14163,7 +14107,7 @@
         <v>MFLOPs</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="G38" s="13">
         <f>'Prefill_8K'!$AF$15</f>
@@ -14176,7 +14120,7 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="14" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="B39" s="14">
         <f>IF(ABS(G39)&gt;=1E15,G39/1E15,IF(ABS(G39)&gt;=1E12,G39/1E12,IF(ABS(G39)&gt;=1E9,G39/1E9,IF(ABS(G39)&gt;=1E6,G39/1E6,G39))))</f>
@@ -14195,7 +14139,7 @@
         <v>GFLOPs</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="G39" s="13">
         <f>'Prefill_8K'!$AF$16</f>
@@ -14208,7 +14152,7 @@
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="4" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="B40" s="12">
         <f>IF(ABS(G40)&gt;=1E12,G40/1E12,IF(ABS(G40)&gt;=1E9,G40/1E9,IF(ABS(G40)&gt;=1E6,G40/1E6,IF(ABS(G40)&gt;=1E3,G40/1E3,G40))))</f>
@@ -14227,7 +14171,7 @@
         <v>GB</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="G40" s="13">
         <f>'Prefill_8K'!$AF$17</f>
@@ -14240,7 +14184,7 @@
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="4" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="B41" s="12">
         <f>IF(ABS(G41)&gt;=1E12,G41/1E12,IF(ABS(G41)&gt;=1E9,G41/1E9,IF(ABS(G41)&gt;=1E6,G41/1E6,IF(ABS(G41)&gt;=1E3,G41/1E3,G41))))</f>
@@ -14259,7 +14203,7 @@
         <v>GB</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="G41" s="13">
         <f>'Prefill_8K'!$AF$18</f>
@@ -14272,7 +14216,7 @@
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="4" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B42" s="12">
         <f>IF(ABS(G42)&gt;=1E12,G42/1E12,IF(ABS(G42)&gt;=1E9,G42/1E9,IF(ABS(G42)&gt;=1E6,G42/1E6,IF(ABS(G42)&gt;=1E3,G42/1E3,G42))))</f>
@@ -14291,7 +14235,7 @@
         <v>MB</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="G42" s="13">
         <f>'Prefill_8K'!$AF$19</f>
@@ -14304,7 +14248,7 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="14" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="B43" s="14">
         <f>IF(ABS(G43)&gt;=1E12,G43/1E12,IF(ABS(G43)&gt;=1E9,G43/1E9,IF(ABS(G43)&gt;=1E6,G43/1E6,IF(ABS(G43)&gt;=1E3,G43/1E3,G43))))</f>
@@ -14323,7 +14267,7 @@
         <v>GB</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="G43" s="13">
         <f>'Prefill_8K'!$AF$20</f>
@@ -14336,7 +14280,7 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="4" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B44" s="12">
         <f>G44</f>
@@ -14353,7 +14297,7 @@
         <v>159</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="G44" s="13">
         <f>'Prefill_8K'!$AF$17/(PrefillTargetMs/1000)/1E9</f>
@@ -14366,7 +14310,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B45" s="12">
         <f>G45</f>
@@ -14383,7 +14327,7 @@
         <v>159</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="G45" s="13">
         <f>'Prefill_8K'!$AF$18/(PrefillTargetMs/1000)/1E9</f>
@@ -14396,7 +14340,7 @@
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="4" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="B46" s="12">
         <f>G46</f>
@@ -14413,7 +14357,7 @@
         <v>159</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="G46" s="13">
         <f>'Prefill_8K'!$AF$19/(PrefillTargetMs/1000)/1E9</f>
@@ -14426,7 +14370,7 @@
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B47" s="12">
         <f>G47</f>
@@ -14443,7 +14387,7 @@
         <v>155</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="G47" s="13">
         <f>'Prefill_8K'!$AF$23</f>
@@ -14456,7 +14400,7 @@
     </row>
     <row r="48" spans="1:8">
       <c r="A48" s="4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B48" s="12">
         <f>IF(ABS(G48)&gt;=1E12,G48/1E12,IF(ABS(G48)&gt;=1E9,G48/1E9,IF(ABS(G48)&gt;=1E6,G48/1E6,IF(ABS(G48)&gt;=1E3,G48/1E3,G48))))</f>
@@ -14475,7 +14419,7 @@
         <v>MB</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="G48" s="13">
         <f>'Prefill_8K'!$AF$21</f>
@@ -14488,7 +14432,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="4" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B49" s="12">
         <f>G49</f>
@@ -14505,7 +14449,7 @@
         <v>159</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="G49" s="13">
         <f>'Prefill_8K'!$AF$21/(PrefillTargetMs/1000)/1E9</f>
@@ -14518,7 +14462,7 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="4" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B50" s="12">
         <f>IF(ABS(G50)&gt;=1E12,G50/1E12,IF(ABS(G50)&gt;=1E9,G50/1E9,IF(ABS(G50)&gt;=1E6,G50/1E6,IF(ABS(G50)&gt;=1E3,G50/1E3,G50))))</f>
@@ -14537,7 +14481,7 @@
         <v>G params</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="G50" s="13">
         <f>'Memory'!$Q$18</f>
@@ -14550,7 +14494,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="4" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B51" s="12">
         <f>IF(ABS(G51)&gt;=1E12,G51/1E12,IF(ABS(G51)&gt;=1E9,G51/1E9,IF(ABS(G51)&gt;=1E6,G51/1E6,IF(ABS(G51)&gt;=1E3,G51/1E3,G51))))</f>
@@ -14569,7 +14513,7 @@
         <v>G params</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="G51" s="13">
         <f>'Memory'!$Q$19</f>
@@ -14582,7 +14526,7 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="4" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B52" s="12">
         <f>IF(ABS(G52)&gt;=1E12,G52/1E12,IF(ABS(G52)&gt;=1E9,G52/1E9,IF(ABS(G52)&gt;=1E6,G52/1E6,IF(ABS(G52)&gt;=1E3,G52/1E3,G52))))</f>
@@ -14601,7 +14545,7 @@
         <v>M params</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="G52" s="13">
         <f>'Memory'!$Q$20</f>
@@ -14614,7 +14558,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="14" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="B53" s="14">
         <f>IF(ABS(G53)&gt;=1E12,G53/1E12,IF(ABS(G53)&gt;=1E9,G53/1E9,IF(ABS(G53)&gt;=1E6,G53/1E6,IF(ABS(G53)&gt;=1E3,G53/1E3,G53))))</f>
@@ -14633,7 +14577,7 @@
         <v>G params</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="G53" s="13">
         <f>'Memory'!$Q$21</f>
@@ -14646,7 +14590,7 @@
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="4" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="B54" s="12">
         <f>IF(ABS(G54)&gt;=1E12,G54/1E12,IF(ABS(G54)&gt;=1E9,G54/1E9,IF(ABS(G54)&gt;=1E6,G54/1E6,IF(ABS(G54)&gt;=1E3,G54/1E3,G54))))</f>
@@ -14665,7 +14609,7 @@
         <v>GB</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="G54" s="13">
         <f>'Memory'!$S$18</f>
@@ -14678,7 +14622,7 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="4" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="B55" s="12">
         <f>IF(ABS(G55)&gt;=1E12,G55/1E12,IF(ABS(G55)&gt;=1E9,G55/1E9,IF(ABS(G55)&gt;=1E6,G55/1E6,IF(ABS(G55)&gt;=1E3,G55/1E3,G55))))</f>
@@ -14697,7 +14641,7 @@
         <v>GB</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="G55" s="13">
         <f>'Memory'!$S$19</f>
@@ -14710,7 +14654,7 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="4" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="B56" s="12">
         <f>IF(ABS(G56)&gt;=1E12,G56/1E12,IF(ABS(G56)&gt;=1E9,G56/1E9,IF(ABS(G56)&gt;=1E6,G56/1E6,IF(ABS(G56)&gt;=1E3,G56/1E3,G56))))</f>
@@ -14729,7 +14673,7 @@
         <v>MB</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="G56" s="13">
         <f>'Memory'!$S$20</f>
@@ -14742,7 +14686,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="14" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="B57" s="14">
         <f>IF(ABS(G57)&gt;=1E12,G57/1E12,IF(ABS(G57)&gt;=1E9,G57/1E9,IF(ABS(G57)&gt;=1E6,G57/1E6,IF(ABS(G57)&gt;=1E3,G57/1E3,G57))))</f>
@@ -14761,7 +14705,7 @@
         <v>GB</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G57" s="13">
         <f>'Memory'!$S$21</f>
@@ -14774,7 +14718,7 @@
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="4" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B58" s="12">
         <f>IF(ABS(G58)&gt;=1E12,G58/1E12,IF(ABS(G58)&gt;=1E9,G58/1E9,IF(ABS(G58)&gt;=1E6,G58/1E6,IF(ABS(G58)&gt;=1E3,G58/1E3,G58))))</f>
@@ -14793,7 +14737,7 @@
         <v>GB</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G58" s="13">
         <f>'Memory'!$Q$26</f>
@@ -14806,7 +14750,7 @@
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="4" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B59" s="12">
         <f>IF(ABS(G59)&gt;=1E12,G59/1E12,IF(ABS(G59)&gt;=1E9,G59/1E9,IF(ABS(G59)&gt;=1E6,G59/1E6,IF(ABS(G59)&gt;=1E3,G59/1E3,G59))))</f>
@@ -14825,7 +14769,7 @@
         <v>GB</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G59" s="13">
         <f>'Memory'!$Q$27</f>
@@ -14838,7 +14782,7 @@
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="4" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B60" s="12">
         <f>IF(ABS(G60)&gt;=1E12,G60/1E12,IF(ABS(G60)&gt;=1E9,G60/1E9,IF(ABS(G60)&gt;=1E6,G60/1E6,IF(ABS(G60)&gt;=1E3,G60/1E3,G60))))</f>
@@ -14857,7 +14801,7 @@
         <v>MB</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G60" s="13">
         <f>'Memory'!$Q$28</f>
@@ -14870,7 +14814,7 @@
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="4" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B61" s="12">
         <f>IF(ABS(G61)&gt;=1E12,G61/1E12,IF(ABS(G61)&gt;=1E9,G61/1E9,IF(ABS(G61)&gt;=1E6,G61/1E6,IF(ABS(G61)&gt;=1E3,G61/1E3,G61))))</f>
@@ -14889,7 +14833,7 @@
         <v>GB</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G61" s="13">
         <f>'Memory'!$Q$29</f>
@@ -14902,7 +14846,7 @@
     </row>
     <row r="62" spans="1:8">
       <c r="A62" s="14" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B62" s="14">
         <f>IF(ABS(G62)&gt;=1E12,G62/1E12,IF(ABS(G62)&gt;=1E9,G62/1E9,IF(ABS(G62)&gt;=1E6,G62/1E6,IF(ABS(G62)&gt;=1E3,G62/1E3,G62))))</f>
@@ -14921,7 +14865,7 @@
         <v>GB</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="G62" s="13">
         <f>'Memory'!$S$21+'Memory'!$Q$29</f>

</xml_diff>

<commit_message>
Adjust calculator chart pair layout
</commit_message>
<xml_diff>
--- a/calculate/deepseek_v4_flash_calculator.xlsx
+++ b/calculate/deepseek_v4_flash_calculator.xlsx
@@ -763,7 +763,7 @@
     <t>在当前场景令牌数下，单个路由专家至少被激活一次的概率，用于估算路由专家参数读取量。</t>
   </si>
   <si>
-    <t>Inference calculation detail</t>
+    <t>推理计算明细</t>
   </si>
   <si>
     <t>Operator/item</t>
@@ -1213,7 +1213,7 @@
     <t>Score routing (FP32)</t>
   </si>
   <si>
-    <t>Parameters and cache: 8K Prefill parameters and capacity</t>
+    <t>参数与缓存：8K 预填充 参数与容量</t>
   </si>
   <si>
     <t>Parameter component</t>
@@ -1294,13 +1294,13 @@
     <t>模型尾部推理参数在每个 Rank 上复制。</t>
   </si>
   <si>
-    <t>Parameter count and capacity summary</t>
+    <t>参数量与参数容量汇总</t>
   </si>
   <si>
     <t>Total</t>
   </si>
   <si>
-    <t>Current scenario KV cache and Compressor state (per Rank, replicated across TP)</t>
+    <t>当前场景 KV 缓存与 Compressor 状态（每 Rank，TP 间复制）</t>
   </si>
   <si>
     <t>Item</t>
@@ -1333,7 +1333,7 @@
     <t>按 MaxContext 为预填充阶段预分配。</t>
   </si>
   <si>
-    <t>Per-rank device resident capacity (default even sharding)</t>
+    <t>单 Rank 设备驻留容量（默认均匀分片）</t>
   </si>
   <si>
     <t>Configuration</t>
@@ -1378,7 +1378,7 @@
     <t>All 8 ranks identical</t>
   </si>
   <si>
-    <t>Parameters and cache: 1M-context Decode parameters and capacity</t>
+    <t>参数与缓存：1M 解码 参数与容量</t>
   </si>
   <si>
     <t>Decode effective main KV</t>
@@ -3210,14 +3210,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
       <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>4705350</xdr:colOff>
       <xdr:row>67</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
@@ -3270,14 +3270,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
       <xdr:row>68</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>4705350</xdr:colOff>
       <xdr:row>84</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
@@ -3330,14 +3330,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
       <xdr:row>85</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>4705350</xdr:colOff>
       <xdr:row>101</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>

</xml_diff>

<commit_message>
Redesign calculator comparison layout
</commit_message>
<xml_diff>
--- a/calculate/deepseek_v4_flash_calculator.xlsx
+++ b/calculate/deepseek_v4_flash_calculator.xlsx
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1465" uniqueCount="558">
   <si>
     <t>DeepSeek V4 Flash - Editable Architecture Parameters</t>
   </si>
@@ -1534,7 +1534,7 @@
     <t>Preallocated KV + state</t>
   </si>
   <si>
-    <t>Total resident capacity</t>
+    <t>Total capacity per inference / rank</t>
   </si>
   <si>
     <t>参数 + 按 MaxContext 预分配的 KV/状态；不含临时工作区。</t>
@@ -1546,6 +1546,30 @@
     <t>单次推理调用的单 Rank 总 FLOPs；不除以目标时延。</t>
   </si>
   <si>
+    <t>Mode</t>
+  </si>
+  <si>
+    <t>TP1</t>
+  </si>
+  <si>
+    <t>TP8/rank</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>Prefill</t>
+  </si>
+  <si>
+    <t>Static parameters + Prefill MaxContext KV/State</t>
+  </si>
+  <si>
+    <t>Decode</t>
+  </si>
+  <si>
+    <t>Static parameters + Decode MaxContext KV/State</t>
+  </si>
+  <si>
     <t>One-inference TFLOPs</t>
   </si>
   <si>
@@ -1576,10 +1600,13 @@
     <t>TP8 GB</t>
   </si>
   <si>
-    <t>Prefill</t>
-  </si>
-  <si>
-    <t>Decode</t>
+    <t>具体内容（Static parameter capacity per rank）：Attention、MoE、Embedding、LM Head、Norm、HC 等静态模型参数及量化 Scale；不含 KV Cache、Compressor State、临时激活和集合通信缓冲区。Prefill/Decode 两图的静态参数数据相同。</t>
+  </si>
+  <si>
+    <t>Capacity GB</t>
+  </si>
+  <si>
+    <t>具体内容（Total capacity per inference / rank）：当前模式单 Rank 的静态参数容量 + 按 MaxContext 预分配的 KV Cache + Compressor State；不含临时激活、residual/HC workspace 和集合通信传输量。</t>
   </si>
   <si>
     <t>Per-Rank Inference Hardware Resource Summary</t>
@@ -1645,9 +1672,6 @@
     <t>Active</t>
   </si>
   <si>
-    <t>Mode</t>
-  </si>
-  <si>
     <t>Attention behavior</t>
   </si>
   <si>
@@ -1667,9 +1691,6 @@
   </si>
   <si>
     <t>Topic</t>
-  </si>
-  <si>
-    <t>Definition</t>
   </si>
   <si>
     <t>仅统计 43 层主推理路径；不含 MTP、反向传播、梯度、优化器状态和训练激活。Layer_Config 最多可维护 64 层。</t>
@@ -2469,7 +2490,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Static parameter capacity per rank</a:t>
+              <a:t>Prefill static parameter capacity per rank</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2651,7 +2672,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>TP1 vs TP8: inference resident capacity per rank</a:t>
+              <a:t>Decode static parameter capacity per rank</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2675,29 +2696,35 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Comparison!$S$60:$S$61</c:f>
+              <c:f>Comparison!$S$60:$S$62</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Prefill</c:v>
+                  <c:v>Attention</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Decode</c:v>
+                  <c:v>MoE</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Other</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Comparison!$T$60:$T$61</c:f>
+              <c:f>Comparison!$T$60:$T$62</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>166.349315548</c:v>
+                  <c:v>7.45138496</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>166.349315548</c:v>
+                  <c:v>148.351461888</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.314423644</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2715,29 +2742,35 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Comparison!$S$60:$S$61</c:f>
+              <c:f>Comparison!$S$60:$S$62</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Prefill</c:v>
+                  <c:v>Attention</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Decode</c:v>
+                  <c:v>MoE</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Other</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Comparison!$U$60:$U$61</c:f>
+              <c:f>Comparison!$U$60:$U$62</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>29.581867388</c:v>
+                  <c:v>2.23750496</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>29.581867388</c:v>
+                  <c:v>19.57794048</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.534376892</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2805,6 +2838,268 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:style val="10"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Prefill total capacity per inference
+/ rank</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Capacity GB</c:v>
+          </c:tx>
+          <c:dLbls>
+            <c:numFmt formatCode="0.0&quot; GB&quot;" sourceLinked="0"/>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Comparison!$S$67:$S$68</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>TP1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>TP8/rank</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Comparison!$T$67:$T$68</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>166.349315548</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>29.581867388</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="30"/>
+        <c:axId val="50060001"/>
+        <c:axId val="50060002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50060001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="low"/>
+        <c:crossAx val="50060002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50060002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>GB</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="0.0&quot; GB&quot;" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50060001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout/>
+    </c:legend>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:style val="10"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Decode total capacity per inference
+/ rank</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Capacity GB</c:v>
+          </c:tx>
+          <c:dLbls>
+            <c:numFmt formatCode="0.0&quot; GB&quot;" sourceLinked="0"/>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Comparison!$S$74:$S$75</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>TP1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>TP8/rank</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Comparison!$T$74:$T$75</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>166.349315548</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>29.581867388</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="30"/>
+        <c:axId val="50070001"/>
+        <c:axId val="50070002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50070001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="low"/>
+        <c:crossAx val="50070002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50070002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>GB</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="0.0&quot; GB&quot;" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50070001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout/>
+    </c:legend>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -2841,13 +3136,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>1038225</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>70</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2871,13 +3166,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>238125</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>4705350</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>70</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2901,13 +3196,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>64</xdr:row>
+      <xdr:row>78</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>1038225</xdr:colOff>
-      <xdr:row>80</xdr:row>
+      <xdr:row>94</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2931,13 +3226,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>238125</xdr:colOff>
-      <xdr:row>64</xdr:row>
+      <xdr:row>78</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>4705350</xdr:colOff>
-      <xdr:row>80</xdr:row>
+      <xdr:row>94</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2952,6 +3247,66 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1038225</xdr:colOff>
+      <xdr:row>118</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>4705350</xdr:colOff>
+      <xdr:row>118</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 7"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3082,6 +3437,19 @@
     <tableColumn id="4" name="Decode TP1"/>
     <tableColumn id="5" name="Decode TP8/rank"/>
     <tableColumn id="6" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Comparison_Total_Capacity" displayName="Comparison_Total_Capacity" ref="K32:N34" totalsRowShown="0">
+  <autoFilter ref="K32:N34"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Mode"/>
+    <tableColumn id="2" name="TP1"/>
+    <tableColumn id="3" name="TP8/rank"/>
+    <tableColumn id="4" name="Definition"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11406,13 +11774,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U61"/>
+  <dimension ref="A1:U121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
     <col min="2" max="5" width="20.7109375" customWidth="1"/>
     <col min="6" max="6" width="72.7109375" customWidth="1"/>
     <col min="7" max="10" width="0" hidden="1" customWidth="1"/>
+    <col min="11" max="14" width="20.7109375" customWidth="1"/>
+    <col min="15" max="16" width="0" hidden="1" customWidth="1"/>
     <col min="19" max="21" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -12407,14 +12777,32 @@
       </c>
     </row>
     <row r="31" spans="1:20">
+      <c r="K31" s="30" t="s">
+        <v>478</v>
+      </c>
+      <c r="L31" s="30"/>
+      <c r="M31" s="30"/>
+      <c r="N31" s="30"/>
       <c r="S31" s="3" t="s">
         <v>2</v>
       </c>
       <c r="T31" s="3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20">
+      <c r="K32" t="s">
         <v>482</v>
       </c>
-    </row>
-    <row r="32" spans="1:20">
+      <c r="L32" t="s">
+        <v>483</v>
+      </c>
+      <c r="M32" t="s">
+        <v>484</v>
+      </c>
+      <c r="N32" t="s">
+        <v>485</v>
+      </c>
       <c r="S32" s="4" t="s">
         <v>439</v>
       </c>
@@ -12423,16 +12811,60 @@
         <v>228.39768211456</v>
       </c>
     </row>
-    <row r="33" spans="19:21">
+    <row r="33" spans="11:21">
+      <c r="K33" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="L33" s="33" t="str">
+        <f>TEXT(IF(ABS(O33)&gt;=1E12,O33/1E12,IF(ABS(O33)&gt;=1E9,O33/1E9,IF(ABS(O33)&gt;=1E6,O33/1E6,IF(ABS(O33)&gt;=1E3,O33/1E3,O33)))),"#,##0.000")&amp;IF((IF(ABS(O33)&gt;=1E12,"TB",IF(ABS(O33)&gt;=1E9,"GB",IF(ABS(O33)&gt;=1E6,"MB",IF(ABS(O33)&gt;=1E3,"KB","bytes")))))="",""," "&amp;(IF(ABS(O33)&gt;=1E12,"TB",IF(ABS(O33)&gt;=1E9,"GB",IF(ABS(O33)&gt;=1E6,"MB",IF(ABS(O33)&gt;=1E3,"KB","bytes"))))))</f>
+        <v>166.349 GB</v>
+      </c>
+      <c r="M33" s="33" t="str">
+        <f>TEXT(IF(ABS(P33)&gt;=1E12,P33/1E12,IF(ABS(P33)&gt;=1E9,P33/1E9,IF(ABS(P33)&gt;=1E6,P33/1E6,IF(ABS(P33)&gt;=1E3,P33/1E3,P33)))),"#,##0.000")&amp;IF((IF(ABS(P33)&gt;=1E12,"TB",IF(ABS(P33)&gt;=1E9,"GB",IF(ABS(P33)&gt;=1E6,"MB",IF(ABS(P33)&gt;=1E3,"KB","bytes")))))="",""," "&amp;(IF(ABS(P33)&gt;=1E12,"TB",IF(ABS(P33)&gt;=1E9,"GB",IF(ABS(P33)&gt;=1E6,"MB",IF(ABS(P33)&gt;=1E3,"KB","bytes"))))))</f>
+        <v>29.582 GB</v>
+      </c>
+      <c r="N33" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="O33" s="32">
+        <f>G27</f>
+        <v>166349315548.0</v>
+      </c>
+      <c r="P33" s="32">
+        <f>H27</f>
+        <v>29581867388.0</v>
+      </c>
       <c r="S33" s="4" t="s">
-        <v>483</v>
+        <v>491</v>
       </c>
       <c r="T33" s="32">
         <f>H28/1e+12</f>
         <v>55.652568907776</v>
       </c>
     </row>
-    <row r="34" spans="19:21">
+    <row r="34" spans="11:21">
+      <c r="K34" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="L34" s="33" t="str">
+        <f>TEXT(IF(ABS(O34)&gt;=1E12,O34/1E12,IF(ABS(O34)&gt;=1E9,O34/1E9,IF(ABS(O34)&gt;=1E6,O34/1E6,IF(ABS(O34)&gt;=1E3,O34/1E3,O34)))),"#,##0.000")&amp;IF((IF(ABS(O34)&gt;=1E12,"TB",IF(ABS(O34)&gt;=1E9,"GB",IF(ABS(O34)&gt;=1E6,"MB",IF(ABS(O34)&gt;=1E3,"KB","bytes")))))="",""," "&amp;(IF(ABS(O34)&gt;=1E12,"TB",IF(ABS(O34)&gt;=1E9,"GB",IF(ABS(O34)&gt;=1E6,"MB",IF(ABS(O34)&gt;=1E3,"KB","bytes"))))))</f>
+        <v>166.349 GB</v>
+      </c>
+      <c r="M34" s="33" t="str">
+        <f>TEXT(IF(ABS(P34)&gt;=1E12,P34/1E12,IF(ABS(P34)&gt;=1E9,P34/1E9,IF(ABS(P34)&gt;=1E6,P34/1E6,IF(ABS(P34)&gt;=1E3,P34/1E3,P34)))),"#,##0.000")&amp;IF((IF(ABS(P34)&gt;=1E12,"TB",IF(ABS(P34)&gt;=1E9,"GB",IF(ABS(P34)&gt;=1E6,"MB",IF(ABS(P34)&gt;=1E3,"KB","bytes")))))="",""," "&amp;(IF(ABS(P34)&gt;=1E12,"TB",IF(ABS(P34)&gt;=1E9,"GB",IF(ABS(P34)&gt;=1E6,"MB",IF(ABS(P34)&gt;=1E3,"KB","bytes"))))))</f>
+        <v>29.582 GB</v>
+      </c>
+      <c r="N34" s="4" t="s">
+        <v>489</v>
+      </c>
+      <c r="O34" s="32">
+        <f>I27</f>
+        <v>166349315548.0</v>
+      </c>
+      <c r="P34" s="32">
+        <f>J27</f>
+        <v>29581867388.0</v>
+      </c>
       <c r="S34" s="4" t="s">
         <v>441</v>
       </c>
@@ -12441,27 +12873,27 @@
         <v>0.14035575211</v>
       </c>
     </row>
-    <row r="35" spans="19:21">
+    <row r="35" spans="11:21">
       <c r="S35" s="4" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
       <c r="T35" s="32">
         <f>J28/1e+12</f>
         <v>0.023549694126</v>
       </c>
     </row>
-    <row r="38" spans="19:21">
+    <row r="38" spans="11:21">
       <c r="S38" s="3" t="s">
         <v>2</v>
       </c>
       <c r="T38" s="3" t="s">
-        <v>485</v>
+        <v>493</v>
       </c>
       <c r="U38" s="3" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="39" spans="19:21">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="39" spans="11:21">
       <c r="S39" s="4" t="s">
         <v>40</v>
       </c>
@@ -12474,7 +12906,7 @@
         <v>23.172382457856</v>
       </c>
     </row>
-    <row r="40" spans="19:21">
+    <row r="40" spans="11:21">
       <c r="S40" s="4" t="s">
         <v>59</v>
       </c>
@@ -12487,9 +12919,9 @@
         <v>31.765578121216</v>
       </c>
     </row>
-    <row r="41" spans="19:21">
+    <row r="41" spans="11:21">
       <c r="S41" s="4" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
       <c r="T41" s="32">
         <f>G7/1e+12</f>
@@ -12500,18 +12932,18 @@
         <v>0.714608328704</v>
       </c>
     </row>
-    <row r="45" spans="19:21">
+    <row r="45" spans="11:21">
       <c r="S45" s="3" t="s">
         <v>2</v>
       </c>
       <c r="T45" s="3" t="s">
-        <v>488</v>
+        <v>496</v>
       </c>
       <c r="U45" s="3" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="46" spans="19:21">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="46" spans="11:21">
       <c r="S46" s="4" t="s">
         <v>40</v>
       </c>
@@ -12524,7 +12956,7 @@
         <v>19.452461056</v>
       </c>
     </row>
-    <row r="47" spans="19:21">
+    <row r="47" spans="11:21">
       <c r="S47" s="4" t="s">
         <v>59</v>
       </c>
@@ -12537,9 +12969,9 @@
         <v>3.877634048</v>
       </c>
     </row>
-    <row r="48" spans="19:21">
+    <row r="48" spans="11:21">
       <c r="S48" s="4" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
       <c r="T48" s="32">
         <f>I7/1e+09</f>
@@ -12555,10 +12987,10 @@
         <v>2</v>
       </c>
       <c r="T52" s="3" t="s">
-        <v>490</v>
+        <v>498</v>
       </c>
       <c r="U52" s="3" t="s">
-        <v>491</v>
+        <v>499</v>
       </c>
     </row>
     <row r="53" spans="19:21">
@@ -12589,7 +13021,7 @@
     </row>
     <row r="55" spans="19:21">
       <c r="S55" s="4" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
       <c r="T55" s="32">
         <f>G21/1e+09</f>
@@ -12605,43 +13037,140 @@
         <v>2</v>
       </c>
       <c r="T59" s="3" t="s">
-        <v>490</v>
+        <v>498</v>
       </c>
       <c r="U59" s="3" t="s">
-        <v>491</v>
+        <v>499</v>
       </c>
     </row>
     <row r="60" spans="19:21">
       <c r="S60" s="4" t="s">
-        <v>492</v>
+        <v>40</v>
       </c>
       <c r="T60" s="32">
+        <f>I19/1e+09</f>
+        <v>7.45138496</v>
+      </c>
+      <c r="U60" s="32">
+        <f>J19/1e+09</f>
+        <v>2.23750496</v>
+      </c>
+    </row>
+    <row r="61" spans="19:21">
+      <c r="S61" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="T61" s="32">
+        <f>I20/1e+09</f>
+        <v>148.351461888</v>
+      </c>
+      <c r="U61" s="32">
+        <f>J20/1e+09</f>
+        <v>19.57794048</v>
+      </c>
+    </row>
+    <row r="62" spans="19:21">
+      <c r="S62" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="T62" s="32">
+        <f>I21/1e+09</f>
+        <v>3.314423644</v>
+      </c>
+      <c r="U62" s="32">
+        <f>J21/1e+09</f>
+        <v>0.534376892</v>
+      </c>
+    </row>
+    <row r="66" spans="19:20">
+      <c r="S66" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="T66" s="3" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="67" spans="19:20">
+      <c r="S67" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="T67" s="32">
         <f>G27/1e+09</f>
         <v>166.349315548</v>
       </c>
-      <c r="U60" s="32">
+    </row>
+    <row r="68" spans="19:20">
+      <c r="S68" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="T68" s="32">
         <f>H27/1e+09</f>
         <v>29.581867388</v>
       </c>
     </row>
-    <row r="61" spans="19:21">
-      <c r="S61" s="4" t="s">
-        <v>493</v>
-      </c>
-      <c r="T61" s="32">
+    <row r="73" spans="19:20">
+      <c r="S73" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="T73" s="3" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="74" spans="19:20">
+      <c r="S74" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="T74" s="32">
         <f>I27/1e+09</f>
         <v>166.349315548</v>
       </c>
-      <c r="U61" s="32">
+    </row>
+    <row r="75" spans="19:20">
+      <c r="S75" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="T75" s="32">
         <f>J27/1e+09</f>
         <v>29.581867388</v>
       </c>
     </row>
+    <row r="97" spans="1:6" ht="36" customHeight="1">
+      <c r="A97" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="B97" s="2"/>
+      <c r="C97" s="2"/>
+      <c r="D97" s="2"/>
+      <c r="E97" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="F97" s="2"/>
+    </row>
+    <row r="121" spans="1:6" ht="36" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="B121" s="2"/>
+      <c r="C121" s="2"/>
+      <c r="D121" s="2"/>
+      <c r="E121" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="F121" s="2"/>
+    </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K31:N31"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="E97:F97"/>
+    <mergeCell ref="A121:D121"/>
+    <mergeCell ref="E121:F121"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12659,17 +13188,17 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>495</v>
+        <v>504</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="30" t="s">
-        <v>496</v>
+        <v>505</v>
       </c>
       <c r="B4" s="30"/>
       <c r="C4" s="30"/>
@@ -12680,10 +13209,10 @@
         <v>438</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>363</v>
@@ -12702,7 +13231,7 @@
         <v>123.969 GFLOPs</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="G6" s="32">
         <f>'Prefill_8K'!$AF$14</f>
@@ -12726,7 +13255,7 @@
         <v>15.240 GFLOPs</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="G7" s="32">
         <f>'Prefill_8K'!$AF$15</f>
@@ -12750,7 +13279,7 @@
         <v>1.146 GFLOPs</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="G8" s="32">
         <f>'Prefill_8K'!$AO$48</f>
@@ -12774,7 +13303,7 @@
         <v>140.356 GFLOPs</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="G9" s="32">
         <f>'Prefill_8K'!$AF$13</f>
@@ -12798,7 +13327,7 @@
         <v>1,049.223 GB/s</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="G10" s="32">
         <f>'Prefill_8K'!$AG$14/(PrefillTargetMs/1000)/1E9</f>
@@ -12822,7 +13351,7 @@
         <v>462.703 GB/s</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="G11" s="32">
         <f>'Prefill_8K'!$AG$15/(PrefillTargetMs/1000)/1E9</f>
@@ -12846,7 +13375,7 @@
         <v>226.865 GB/s</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="G12" s="32">
         <f>'Prefill_8K'!$AQ$48/(PrefillTargetMs/1000)/1E9</f>
@@ -12870,7 +13399,7 @@
         <v>140.356 GFLOPs</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>501</v>
+        <v>510</v>
       </c>
       <c r="G13" s="32">
         <f>'Prefill_8K'!$AF$13</f>
@@ -12894,7 +13423,7 @@
         <v>0.000 B</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="G14" s="32">
         <f>'Prefill_8K'!$AS$48</f>
@@ -12942,7 +13471,7 @@
         <v>5.086 G</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="G16" s="32">
         <f>'Prefill_8K'!$AY$49</f>
@@ -12990,7 +13519,7 @@
         <v>1.093 G</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="G18" s="32">
         <f>'Prefill_8K'!$AY$51</f>
@@ -13014,7 +13543,7 @@
         <v>284.335 G</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="G19" s="32">
         <f>'Prefill_8K'!$AY$52</f>
@@ -13038,7 +13567,7 @@
         <v>7.451 GB</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="G20" s="32">
         <f>'Prefill_8K'!$BA$49</f>
@@ -13062,7 +13591,7 @@
         <v>148.351 GB</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>507</v>
+        <v>516</v>
       </c>
       <c r="G21" s="32">
         <f>'Prefill_8K'!$BA$50</f>
@@ -13086,7 +13615,7 @@
         <v>3.314 GB</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="G22" s="32">
         <f>'Prefill_8K'!$BA$51</f>
@@ -13110,7 +13639,7 @@
         <v>159.117 GB</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>508</v>
+        <v>517</v>
       </c>
       <c r="G23" s="32">
         <f>'Prefill_8K'!$BA$52</f>
@@ -13134,7 +13663,7 @@
         <v>5.811 GB</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="G24" s="32">
         <f>'Prefill_8K'!$U$35</f>
@@ -13158,7 +13687,7 @@
         <v>1.409 GB</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="G25" s="32">
         <f>'Prefill_8K'!$U$36</f>
@@ -13182,7 +13711,7 @@
         <v>12.206 MB</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="G26" s="32">
         <f>'Prefill_8K'!$U$37</f>
@@ -13206,7 +13735,7 @@
         <v>7.232 GB</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="G27" s="32">
         <f>'Prefill_8K'!$U$38</f>
@@ -13230,7 +13759,7 @@
         <v>166.349 GB</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>510</v>
+        <v>519</v>
       </c>
       <c r="G28" s="32">
         <f>'Prefill_8K'!$BA$52+'Prefill_8K'!$U$38</f>
@@ -13243,7 +13772,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="30" t="s">
-        <v>511</v>
+        <v>520</v>
       </c>
       <c r="B30" s="30"/>
       <c r="C30" s="30"/>
@@ -13254,10 +13783,10 @@
         <v>438</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>363</v>
@@ -13276,7 +13805,7 @@
         <v>19.452 GFLOPs</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="G32" s="32">
         <f>'Prefill_8K'!$AI$14</f>
@@ -13300,7 +13829,7 @@
         <v>3.878 GFLOPs</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="G33" s="32">
         <f>'Prefill_8K'!$AI$15</f>
@@ -13324,7 +13853,7 @@
         <v>219.599 MFLOPs</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="G34" s="32">
         <f>'Prefill_8K'!$AP$48</f>
@@ -13348,7 +13877,7 @@
         <v>23.550 GFLOPs</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="G35" s="32">
         <f>'Prefill_8K'!$AI$13</f>
@@ -13372,7 +13901,7 @@
         <v>403.523 GB/s</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="G36" s="32">
         <f>'Prefill_8K'!$AJ$14/(PrefillTargetMs/1000)/1E9</f>
@@ -13396,7 +13925,7 @@
         <v>160.521 GB/s</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="G37" s="32">
         <f>'Prefill_8K'!$AJ$15/(PrefillTargetMs/1000)/1E9</f>
@@ -13420,7 +13949,7 @@
         <v>41.483 GB/s</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="G38" s="32">
         <f>'Prefill_8K'!$AR$48/(PrefillTargetMs/1000)/1E9</f>
@@ -13444,7 +13973,7 @@
         <v>23.550 GFLOPs</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>501</v>
+        <v>510</v>
       </c>
       <c r="G39" s="32">
         <f>'Prefill_8K'!$AI$13</f>
@@ -13468,7 +13997,7 @@
         <v>5.865 MB</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="G40" s="32">
         <f>'Prefill_8K'!$AT$48</f>
@@ -13516,7 +14045,7 @@
         <v>1.140 G</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="G42" s="32">
         <f>'Prefill_8K'!$AZ$49</f>
@@ -13564,7 +14093,7 @@
         <v>166.690 M</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="G44" s="32">
         <f>'Prefill_8K'!$AZ$51</f>
@@ -13588,7 +14117,7 @@
         <v>37.064 G</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="G45" s="32">
         <f>'Prefill_8K'!$AZ$52</f>
@@ -13612,7 +14141,7 @@
         <v>2.238 GB</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="G46" s="32">
         <f>'Prefill_8K'!$BB$49</f>
@@ -13636,7 +14165,7 @@
         <v>19.578 GB</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>507</v>
+        <v>516</v>
       </c>
       <c r="G47" s="32">
         <f>'Prefill_8K'!$BB$50</f>
@@ -13660,7 +14189,7 @@
         <v>534.377 MB</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="G48" s="32">
         <f>'Prefill_8K'!$BB$51</f>
@@ -13684,7 +14213,7 @@
         <v>22.350 GB</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>508</v>
+        <v>517</v>
       </c>
       <c r="G49" s="32">
         <f>'Prefill_8K'!$BB$52</f>
@@ -13708,7 +14237,7 @@
         <v>5.811 GB</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="G50" s="32">
         <f>'Prefill_8K'!$X$35</f>
@@ -13732,7 +14261,7 @@
         <v>1.409 GB</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="G51" s="32">
         <f>'Prefill_8K'!$X$36</f>
@@ -13756,7 +14285,7 @@
         <v>12.206 MB</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="G52" s="32">
         <f>'Prefill_8K'!$X$37</f>
@@ -13780,7 +14309,7 @@
         <v>7.232 GB</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="G53" s="32">
         <f>'Prefill_8K'!$X$38</f>
@@ -13804,7 +14333,7 @@
         <v>29.582 GB</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>510</v>
+        <v>519</v>
       </c>
       <c r="G54" s="32">
         <f>'Prefill_8K'!$BB$52+'Prefill_8K'!$X$38</f>
@@ -13836,12 +14365,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>512</v>
+        <v>521</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>513</v>
+        <v>522</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -13849,19 +14378,19 @@
         <v>421</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>514</v>
+        <v>523</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>515</v>
+        <v>482</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>423</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>516</v>
+        <v>524</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -13872,7 +14401,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D4" s="36">
         <f>IF(C4="window",0,IF(C4="short",ShortRatio,LongRatio))</f>
@@ -13895,7 +14424,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D5" s="36">
         <f>IF(C5="window",0,IF(C5="short",ShortRatio,LongRatio))</f>
@@ -13918,7 +14447,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D6" s="36">
         <f>IF(C6="window",0,IF(C6="short",ShortRatio,LongRatio))</f>
@@ -13941,7 +14470,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D7" s="36">
         <f>IF(C7="window",0,IF(C7="short",ShortRatio,LongRatio))</f>
@@ -13964,7 +14493,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D8" s="36">
         <f>IF(C8="window",0,IF(C8="short",ShortRatio,LongRatio))</f>
@@ -13987,7 +14516,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D9" s="36">
         <f>IF(C9="window",0,IF(C9="short",ShortRatio,LongRatio))</f>
@@ -14010,7 +14539,7 @@
         <v>1</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D10" s="36">
         <f>IF(C10="window",0,IF(C10="short",ShortRatio,LongRatio))</f>
@@ -14033,7 +14562,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D11" s="36">
         <f>IF(C11="window",0,IF(C11="short",ShortRatio,LongRatio))</f>
@@ -14056,7 +14585,7 @@
         <v>1</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D12" s="36">
         <f>IF(C12="window",0,IF(C12="short",ShortRatio,LongRatio))</f>
@@ -14079,7 +14608,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D13" s="36">
         <f>IF(C13="window",0,IF(C13="short",ShortRatio,LongRatio))</f>
@@ -14102,7 +14631,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D14" s="36">
         <f>IF(C14="window",0,IF(C14="short",ShortRatio,LongRatio))</f>
@@ -14125,7 +14654,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D15" s="36">
         <f>IF(C15="window",0,IF(C15="short",ShortRatio,LongRatio))</f>
@@ -14148,7 +14677,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D16" s="36">
         <f>IF(C16="window",0,IF(C16="short",ShortRatio,LongRatio))</f>
@@ -14171,7 +14700,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D17" s="36">
         <f>IF(C17="window",0,IF(C17="short",ShortRatio,LongRatio))</f>
@@ -14194,7 +14723,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D18" s="36">
         <f>IF(C18="window",0,IF(C18="short",ShortRatio,LongRatio))</f>
@@ -14217,7 +14746,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D19" s="36">
         <f>IF(C19="window",0,IF(C19="short",ShortRatio,LongRatio))</f>
@@ -14240,7 +14769,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D20" s="36">
         <f>IF(C20="window",0,IF(C20="short",ShortRatio,LongRatio))</f>
@@ -14263,7 +14792,7 @@
         <v>1</v>
       </c>
       <c r="C21" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D21" s="36">
         <f>IF(C21="window",0,IF(C21="short",ShortRatio,LongRatio))</f>
@@ -14286,7 +14815,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D22" s="36">
         <f>IF(C22="window",0,IF(C22="short",ShortRatio,LongRatio))</f>
@@ -14309,7 +14838,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D23" s="36">
         <f>IF(C23="window",0,IF(C23="short",ShortRatio,LongRatio))</f>
@@ -14332,7 +14861,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D24" s="36">
         <f>IF(C24="window",0,IF(C24="short",ShortRatio,LongRatio))</f>
@@ -14355,7 +14884,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D25" s="36">
         <f>IF(C25="window",0,IF(C25="short",ShortRatio,LongRatio))</f>
@@ -14378,7 +14907,7 @@
         <v>1</v>
       </c>
       <c r="C26" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D26" s="36">
         <f>IF(C26="window",0,IF(C26="short",ShortRatio,LongRatio))</f>
@@ -14401,7 +14930,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D27" s="36">
         <f>IF(C27="window",0,IF(C27="short",ShortRatio,LongRatio))</f>
@@ -14424,7 +14953,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D28" s="36">
         <f>IF(C28="window",0,IF(C28="short",ShortRatio,LongRatio))</f>
@@ -14447,7 +14976,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D29" s="36">
         <f>IF(C29="window",0,IF(C29="short",ShortRatio,LongRatio))</f>
@@ -14470,7 +14999,7 @@
         <v>1</v>
       </c>
       <c r="C30" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D30" s="36">
         <f>IF(C30="window",0,IF(C30="short",ShortRatio,LongRatio))</f>
@@ -14493,7 +15022,7 @@
         <v>1</v>
       </c>
       <c r="C31" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D31" s="36">
         <f>IF(C31="window",0,IF(C31="short",ShortRatio,LongRatio))</f>
@@ -14516,7 +15045,7 @@
         <v>1</v>
       </c>
       <c r="C32" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D32" s="36">
         <f>IF(C32="window",0,IF(C32="short",ShortRatio,LongRatio))</f>
@@ -14539,7 +15068,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D33" s="36">
         <f>IF(C33="window",0,IF(C33="short",ShortRatio,LongRatio))</f>
@@ -14562,7 +15091,7 @@
         <v>1</v>
       </c>
       <c r="C34" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D34" s="36">
         <f>IF(C34="window",0,IF(C34="short",ShortRatio,LongRatio))</f>
@@ -14585,7 +15114,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D35" s="36">
         <f>IF(C35="window",0,IF(C35="short",ShortRatio,LongRatio))</f>
@@ -14608,7 +15137,7 @@
         <v>1</v>
       </c>
       <c r="C36" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D36" s="36">
         <f>IF(C36="window",0,IF(C36="short",ShortRatio,LongRatio))</f>
@@ -14631,7 +15160,7 @@
         <v>1</v>
       </c>
       <c r="C37" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D37" s="36">
         <f>IF(C37="window",0,IF(C37="short",ShortRatio,LongRatio))</f>
@@ -14654,7 +15183,7 @@
         <v>1</v>
       </c>
       <c r="C38" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D38" s="36">
         <f>IF(C38="window",0,IF(C38="short",ShortRatio,LongRatio))</f>
@@ -14677,7 +15206,7 @@
         <v>1</v>
       </c>
       <c r="C39" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D39" s="36">
         <f>IF(C39="window",0,IF(C39="short",ShortRatio,LongRatio))</f>
@@ -14700,7 +15229,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D40" s="36">
         <f>IF(C40="window",0,IF(C40="short",ShortRatio,LongRatio))</f>
@@ -14723,7 +15252,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D41" s="36">
         <f>IF(C41="window",0,IF(C41="short",ShortRatio,LongRatio))</f>
@@ -14746,7 +15275,7 @@
         <v>1</v>
       </c>
       <c r="C42" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D42" s="36">
         <f>IF(C42="window",0,IF(C42="short",ShortRatio,LongRatio))</f>
@@ -14769,7 +15298,7 @@
         <v>1</v>
       </c>
       <c r="C43" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D43" s="36">
         <f>IF(C43="window",0,IF(C43="short",ShortRatio,LongRatio))</f>
@@ -14792,7 +15321,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D44" s="36">
         <f>IF(C44="window",0,IF(C44="short",ShortRatio,LongRatio))</f>
@@ -14815,7 +15344,7 @@
         <v>1</v>
       </c>
       <c r="C45" s="35" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D45" s="36">
         <f>IF(C45="window",0,IF(C45="short",ShortRatio,LongRatio))</f>
@@ -14838,7 +15367,7 @@
         <v>1</v>
       </c>
       <c r="C46" s="35" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="D46" s="36">
         <f>IF(C46="window",0,IF(C46="short",ShortRatio,LongRatio))</f>
@@ -14861,7 +15390,7 @@
         <v>0</v>
       </c>
       <c r="C47" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D47" s="36">
         <f>IF(C47="window",0,IF(C47="short",ShortRatio,LongRatio))</f>
@@ -14884,7 +15413,7 @@
         <v>0</v>
       </c>
       <c r="C48" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D48" s="36">
         <f>IF(C48="window",0,IF(C48="short",ShortRatio,LongRatio))</f>
@@ -14907,7 +15436,7 @@
         <v>0</v>
       </c>
       <c r="C49" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D49" s="36">
         <f>IF(C49="window",0,IF(C49="short",ShortRatio,LongRatio))</f>
@@ -14930,7 +15459,7 @@
         <v>0</v>
       </c>
       <c r="C50" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D50" s="36">
         <f>IF(C50="window",0,IF(C50="short",ShortRatio,LongRatio))</f>
@@ -14953,7 +15482,7 @@
         <v>0</v>
       </c>
       <c r="C51" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D51" s="36">
         <f>IF(C51="window",0,IF(C51="short",ShortRatio,LongRatio))</f>
@@ -14976,7 +15505,7 @@
         <v>0</v>
       </c>
       <c r="C52" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D52" s="36">
         <f>IF(C52="window",0,IF(C52="short",ShortRatio,LongRatio))</f>
@@ -14999,7 +15528,7 @@
         <v>0</v>
       </c>
       <c r="C53" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D53" s="36">
         <f>IF(C53="window",0,IF(C53="short",ShortRatio,LongRatio))</f>
@@ -15022,7 +15551,7 @@
         <v>0</v>
       </c>
       <c r="C54" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D54" s="36">
         <f>IF(C54="window",0,IF(C54="short",ShortRatio,LongRatio))</f>
@@ -15045,7 +15574,7 @@
         <v>0</v>
       </c>
       <c r="C55" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D55" s="36">
         <f>IF(C55="window",0,IF(C55="short",ShortRatio,LongRatio))</f>
@@ -15068,7 +15597,7 @@
         <v>0</v>
       </c>
       <c r="C56" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D56" s="36">
         <f>IF(C56="window",0,IF(C56="short",ShortRatio,LongRatio))</f>
@@ -15091,7 +15620,7 @@
         <v>0</v>
       </c>
       <c r="C57" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D57" s="36">
         <f>IF(C57="window",0,IF(C57="short",ShortRatio,LongRatio))</f>
@@ -15114,7 +15643,7 @@
         <v>0</v>
       </c>
       <c r="C58" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D58" s="36">
         <f>IF(C58="window",0,IF(C58="short",ShortRatio,LongRatio))</f>
@@ -15137,7 +15666,7 @@
         <v>0</v>
       </c>
       <c r="C59" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D59" s="36">
         <f>IF(C59="window",0,IF(C59="short",ShortRatio,LongRatio))</f>
@@ -15160,7 +15689,7 @@
         <v>0</v>
       </c>
       <c r="C60" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D60" s="36">
         <f>IF(C60="window",0,IF(C60="short",ShortRatio,LongRatio))</f>
@@ -15183,7 +15712,7 @@
         <v>0</v>
       </c>
       <c r="C61" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D61" s="36">
         <f>IF(C61="window",0,IF(C61="short",ShortRatio,LongRatio))</f>
@@ -15206,7 +15735,7 @@
         <v>0</v>
       </c>
       <c r="C62" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D62" s="36">
         <f>IF(C62="window",0,IF(C62="short",ShortRatio,LongRatio))</f>
@@ -15229,7 +15758,7 @@
         <v>0</v>
       </c>
       <c r="C63" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D63" s="36">
         <f>IF(C63="window",0,IF(C63="short",ShortRatio,LongRatio))</f>
@@ -15252,7 +15781,7 @@
         <v>0</v>
       </c>
       <c r="C64" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D64" s="36">
         <f>IF(C64="window",0,IF(C64="short",ShortRatio,LongRatio))</f>
@@ -15275,7 +15804,7 @@
         <v>0</v>
       </c>
       <c r="C65" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D65" s="36">
         <f>IF(C65="window",0,IF(C65="short",ShortRatio,LongRatio))</f>
@@ -15298,7 +15827,7 @@
         <v>0</v>
       </c>
       <c r="C66" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D66" s="36">
         <f>IF(C66="window",0,IF(C66="short",ShortRatio,LongRatio))</f>
@@ -15321,7 +15850,7 @@
         <v>0</v>
       </c>
       <c r="C67" s="35" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="D67" s="36">
         <f>IF(C67="window",0,IF(C67="short",ShortRatio,LongRatio))</f>
@@ -15361,15 +15890,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="3" t="s">
-        <v>522</v>
+        <v>530</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>523</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -15377,31 +15906,31 @@
         <v>359</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="4" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="4" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="4" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -15409,39 +15938,39 @@
         <v>59</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>533</v>
+        <v>540</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="4" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4" t="s">
-        <v>536</v>
+        <v>543</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="4" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>539</v>
+        <v>546</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -15449,47 +15978,47 @@
         <v>409</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>540</v>
+        <v>547</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="4" t="s">
-        <v>541</v>
+        <v>548</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="4" t="s">
-        <v>543</v>
+        <v>550</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4" t="s">
-        <v>545</v>
+        <v>552</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="4" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="4" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>550</v>
+        <v>557</v>
       </c>
     </row>
   </sheetData>

</xml_diff>